<commit_message>
Route final summaries by template and fix KDL1 sync
</commit_message>
<xml_diff>
--- a/templates/KB_Market_Improvement_XLSForm.xlsx
+++ b/templates/KB_Market_Improvement_XLSForm.xlsx
@@ -2,599 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rbd6b4fdfb5cd4601"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Reac511fdbad940af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rd643fffe26b44ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="Rade2c1390c0343ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="Rf8f599f0d6f44c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R11e96f0a09964e33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rdf62acb5e3b840a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R8c5fb8d98d7043bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="R0e2639823482489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="Ra0a1d28ebefd4ce5"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t xml:space="preserve">list_name</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">name</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">label</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">region</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">r8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">dealer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">avg4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AVG4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">bke7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BKE7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">bmc2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BMC2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">btb1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BTB1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">bti6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BTI6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">bty8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BTY8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">bvl6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BVL6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ca9</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CA9</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">chk6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CHK6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cks1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CKS1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cph2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CPH2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cuk7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CUK7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kcg4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KCG4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kcm1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KCM1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kd1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KDL1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kht3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KHT3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kkg3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KKG3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">tpg2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TPG2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kps7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KPS7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kpt2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KPT2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">krg7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KRG7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">krt1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KRT1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">krv5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KRV5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ksa5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KSA5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ksm1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KSM1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ksp3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KSP3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ksv5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KSV5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ktb1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KTB1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">kth2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KTH2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ktl6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KTL6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ktm8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KTM8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ktr4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">KTR4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">mdk2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MDK2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">mmt3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MMT3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">mrs5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MRS5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">pkb4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PKB4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">pln4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PLN4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">pmr5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PMR5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">pnp6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PNP6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ppr8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PPR8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ppt3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PPT3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ptm6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PTM6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">puk7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PUK7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">pus5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PUS5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">pvh3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PVH3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">rtk4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">RTK4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">smr5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SMR5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">snl6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SNL6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">sra5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SRA5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">srp1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SRP1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">str3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">STR3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">stt4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">STT4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">sva7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SVA7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">svr4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SVR4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">tak2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TAK2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">tkm2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TKM2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">vvg1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">VVG1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">outlet_type</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">wholesale</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Wholesale</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">drink_shop</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Drink Shop</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">wet_market</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Wet Market</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">trolley</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Trolley</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">yes_no</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">yes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Yes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">no</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">No</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">stock_status</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">full</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">គ្រប់</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">low</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ខ្វះ</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">no_stock</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ដាច់ស្តុក</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">movement_score</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">no_sale</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">អត់មានលក់</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">sale</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">មានលក់</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">fast_sale</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">លក់ដាច់</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ring_pull_in_outlet_choices</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cbl_ncp_6_can</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CBL NCP 6 Can</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cbl_ncp_5_usd</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CBL NCP 5 USD</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">local_eat</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Local Eat</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">coffee_bakery</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Coffee,Bakery</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">canteen</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Canteen</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">sport_club</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sport Club</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">motor_shop</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Motor Shop</x:t>
-  </x:si>
   <x:si>
     <x:t xml:space="preserve">form_title</x:t>
   </x:si>
@@ -13330,13 +12748,13 @@
         <x:v>summary_instruction</x:v>
       </x:c>
       <x:c r="C488" s="1" t="str">
-        <x:v>KEY ISSUES &amp; INITIATIVE IDEA / SUGGESTION — available for every outlet</x:v>
+        <x:v>FINAL KEY ISSUES &amp; INITIATIVE IDEA / SUGGESTION</x:v>
       </x:c>
       <x:c r="D488" s="1" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="E488" s="1" t="str">
-        <x:v>Normal outlet: enter outlet-specific comments if needed; the bot stores them but does not put them in the final summary. Final summary: set Outlet Name to one accepted keyword; the bot copies only that latest row into the report.</x:v>
+        <x:v>Set Outlet Name to an accepted summary keyword. Leave Summary Template blank for GENERAL, or select CHANNEL SPECIALIST for the Channel Specialist report. Then enter up to 4 Key Issues and 4 Initiative/Suggestion points.</x:v>
       </x:c>
       <x:c r="F488" s="1"/>
       <x:c r="G488" s="1"/>
@@ -13347,25 +12765,27 @@
     </x:row>
     <x:row r="489" ht="319">
       <x:c r="A489" s="1" t="str">
-        <x:v>text</x:v>
+        <x:v>select_one summary_report_type</x:v>
       </x:c>
       <x:c r="B489" s="1" t="str">
-        <x:v>key_issues_detail</x:v>
+        <x:v>final_summary_report_type</x:v>
       </x:c>
       <x:c r="C489" s="1" t="str">
-        <x:v>Key Issues Detail</x:v>
+        <x:v>Summary Template / ប្រភេទរបាយការណ៍</x:v>
       </x:c>
       <x:c r="D489" s="1" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="E489" s="1" t="str">
+        <x:v>Leave blank for GENERAL. Select CHANNEL SPECIALIST only when this final summary belongs to the Channel Specialist template.</x:v>
+      </x:c>
+      <x:c r="F489" s="1" t="str">
+        <x:v>minimal</x:v>
+      </x:c>
+      <x:c r="G489" s="1"/>
+      <x:c r="H489" s="1" t="str">
         <x:v>normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'</x:v>
       </x:c>
-      <x:c r="E489" s="1" t="str">
-        <x:v>For a normal outlet, write its Key Issue or leave blank. For the final summary outlet name, write up to 4 combined Key Issues.</x:v>
-      </x:c>
-      <x:c r="F489" s="1" t="str">
-        <x:v>multiline</x:v>
-      </x:c>
-      <x:c r="G489" s="1"/>
-      <x:c r="H489" s="1"/>
       <x:c r="I489" s="1"/>
       <x:c r="J489" s="1"/>
       <x:c r="K489" s="1"/>
@@ -13375,16 +12795,16 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B490" s="1" t="str">
-        <x:v>initiative_idea_suggestion</x:v>
+        <x:v>key_issues_detail</x:v>
       </x:c>
       <x:c r="C490" s="1" t="str">
-        <x:v>Initiative Idea / Suggestion</x:v>
+        <x:v>Key Issues Detail</x:v>
       </x:c>
       <x:c r="D490" s="1" t="str">
         <x:v>normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'</x:v>
       </x:c>
       <x:c r="E490" s="1" t="str">
-        <x:v>For a normal outlet, write its Initiative/Suggestion or leave blank. For the final summary outlet name, write up to 4 combined actions.</x:v>
+        <x:v>For a normal outlet, write its Key Issue or leave blank. For the final summary outlet name, write up to 4 combined Key Issues.</x:v>
       </x:c>
       <x:c r="F490" s="1" t="str">
         <x:v>multiline</x:v>
@@ -13397,20 +12817,45 @@
     </x:row>
     <x:row r="491">
       <x:c r="A491" s="1" t="str">
-        <x:v>end_group</x:v>
-      </x:c>
-      <x:c r="B491" s="1"/>
-      <x:c r="C491" s="1"/>
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B491" s="1" t="str">
+        <x:v>initiative_idea_suggestion</x:v>
+      </x:c>
+      <x:c r="C491" s="1" t="str">
+        <x:v>Initiative Idea / Suggestion</x:v>
+      </x:c>
       <x:c r="D491" s="1" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="E491" s="1"/>
-      <x:c r="F491" s="1"/>
+        <x:v>normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'</x:v>
+      </x:c>
+      <x:c r="E491" s="1" t="str">
+        <x:v>For a normal outlet, write its Initiative/Suggestion or leave blank. For the final summary outlet name, write up to 4 combined actions.</x:v>
+      </x:c>
+      <x:c r="F491" s="1" t="str">
+        <x:v>multiline</x:v>
+      </x:c>
       <x:c r="G491" s="1"/>
       <x:c r="H491" s="1"/>
       <x:c r="I491" s="1"/>
       <x:c r="J491" s="1"/>
       <x:c r="K491" s="1"/>
+    </x:row>
+    <x:row r="492">
+      <x:c r="A492" t="str">
+        <x:v>end_group</x:v>
+      </x:c>
+      <x:c r="B492"/>
+      <x:c r="C492"/>
+      <x:c r="D492" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="E492"/>
+      <x:c r="F492"/>
+      <x:c r="G492"/>
+      <x:c r="H492"/>
+      <x:c r="I492"/>
+      <x:c r="J492"/>
+      <x:c r="K492"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13422,1245 +12867,1264 @@
   <x:sheetFormatPr defaultRowHeight="14.5"/>
   <x:sheetData>
     <x:row r="1" ht="5.75" customHeight="1">
-      <x:c r="A1" s="2" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="s">
-        <x:v>3</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>list_name</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="str">
+        <x:v>label</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="str">
+        <x:v>region</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>5</x:v>
+      <x:c r="A2" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="str">
+        <x:v>r1</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="str">
+        <x:v>R1</x:v>
       </x:c>
       <x:c r="D2" s="1"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="1" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C3" s="1" t="s">
-        <x:v>7</x:v>
+      <x:c r="A3" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="str">
+        <x:v>r2</x:v>
+      </x:c>
+      <x:c r="C3" s="1" t="str">
+        <x:v>R2</x:v>
       </x:c>
       <x:c r="D3" s="1"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B4" s="1" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C4" s="1" t="s">
-        <x:v>9</x:v>
+      <x:c r="A4" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="str">
+        <x:v>r3</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="str">
+        <x:v>R3</x:v>
       </x:c>
       <x:c r="D4" s="1"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="1" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C5" s="1" t="s">
-        <x:v>11</x:v>
+      <x:c r="A5" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="str">
+        <x:v>r4</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="str">
+        <x:v>R4</x:v>
       </x:c>
       <x:c r="D5" s="1"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B6" s="1" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C6" s="1" t="s">
-        <x:v>13</x:v>
+      <x:c r="A6" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="str">
+        <x:v>r5</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="str">
+        <x:v>R5</x:v>
       </x:c>
       <x:c r="D6" s="1"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>15</x:v>
+      <x:c r="A7" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="str">
+        <x:v>r6</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="str">
+        <x:v>R6</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B8" s="1" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C8" s="1" t="s">
-        <x:v>17</x:v>
+      <x:c r="A8" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="str">
+        <x:v>r7</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="str">
+        <x:v>R7</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B9" s="1" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C9" s="1" t="s">
-        <x:v>19</x:v>
+      <x:c r="A9" s="1" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="str">
+        <x:v>r8</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="str">
+        <x:v>R8</x:v>
       </x:c>
       <x:c r="D9" s="1"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="D10" s="1" t="s">
-        <x:v>18</x:v>
+      <x:c r="A10" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="str">
+        <x:v>avg4</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="str">
+        <x:v>AVG4</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="str">
+        <x:v>r8</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B11" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C11" s="1" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D11" s="1" t="s">
-        <x:v>16</x:v>
+      <x:c r="A11" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B11" s="1" t="str">
+        <x:v>bke7</x:v>
+      </x:c>
+      <x:c r="C11" s="1" t="str">
+        <x:v>BKE7</x:v>
+      </x:c>
+      <x:c r="D11" s="1" t="str">
+        <x:v>r7</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B12" s="1" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="C12" s="1" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D12" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A12" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B12" s="1" t="str">
+        <x:v>bmc2</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="str">
+        <x:v>BMC2</x:v>
+      </x:c>
+      <x:c r="D12" s="1" t="str">
+        <x:v>r5</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B13" s="1" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C13" s="1" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="D13" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A13" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B13" s="1" t="str">
+        <x:v>btb1</x:v>
+      </x:c>
+      <x:c r="C13" s="1" t="str">
+        <x:v>BTB1</x:v>
+      </x:c>
+      <x:c r="D13" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B14" s="1" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="C14" s="1" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="D14" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A14" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B14" s="1" t="str">
+        <x:v>bti6</x:v>
+      </x:c>
+      <x:c r="C14" s="1" t="str">
+        <x:v>BTI6</x:v>
+      </x:c>
+      <x:c r="D14" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B15" s="1" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="C15" s="1" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="D15" s="1" t="s">
-        <x:v>14</x:v>
+      <x:c r="A15" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B15" s="1" t="str">
+        <x:v>bty8</x:v>
+      </x:c>
+      <x:c r="C15" s="1" t="str">
+        <x:v>BTY8</x:v>
+      </x:c>
+      <x:c r="D15" s="1" t="str">
+        <x:v>r6</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B16" s="1" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C16" s="1" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D16" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A16" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B16" s="1" t="str">
+        <x:v>bvl6</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="str">
+        <x:v>BVL6</x:v>
+      </x:c>
+      <x:c r="D16" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B17" s="1" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="C17" s="1" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="D17" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A17" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B17" s="1" t="str">
+        <x:v>ca1</x:v>
+      </x:c>
+      <x:c r="C17" s="1" t="str">
+        <x:v>CA1</x:v>
+      </x:c>
+      <x:c r="D17" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B18" s="1" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="C18" s="1" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="D18" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A18" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B18" s="1" t="str">
+        <x:v>ca2</x:v>
+      </x:c>
+      <x:c r="C18" s="1" t="str">
+        <x:v>CA2</x:v>
+      </x:c>
+      <x:c r="D18" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B19" s="1" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="C19" s="1" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="D19" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A19" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B19" s="1" t="str">
+        <x:v>ca3</x:v>
+      </x:c>
+      <x:c r="C19" s="1" t="str">
+        <x:v>CA3</x:v>
+      </x:c>
+      <x:c r="D19" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B20" s="1" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="C20" s="1" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="D20" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A20" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B20" s="1" t="str">
+        <x:v>ca4</x:v>
+      </x:c>
+      <x:c r="C20" s="1" t="str">
+        <x:v>CA4</x:v>
+      </x:c>
+      <x:c r="D20" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B21" s="1" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C21" s="1" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D21" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A21" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B21" s="1" t="str">
+        <x:v>ca5</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="str">
+        <x:v>CA5</x:v>
+      </x:c>
+      <x:c r="D21" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B22" s="1" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="C22" s="1" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="D22" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A22" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B22" s="1" t="str">
+        <x:v>ca6</x:v>
+      </x:c>
+      <x:c r="C22" s="1" t="str">
+        <x:v>CA6</x:v>
+      </x:c>
+      <x:c r="D22" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B23" s="1" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="C23" s="1" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D23" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A23" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B23" s="1" t="str">
+        <x:v>ca7</x:v>
+      </x:c>
+      <x:c r="C23" s="1" t="str">
+        <x:v>CA7</x:v>
+      </x:c>
+      <x:c r="D23" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B24" s="1" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="C24" s="1" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="D24" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A24" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B24" s="1" t="str">
+        <x:v>ca8</x:v>
+      </x:c>
+      <x:c r="C24" s="1" t="str">
+        <x:v>CA8</x:v>
+      </x:c>
+      <x:c r="D24" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B25" s="1" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="C25" s="1" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="D25" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A25" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B25" s="1" t="str">
+        <x:v>ca9</x:v>
+      </x:c>
+      <x:c r="C25" s="1" t="str">
+        <x:v>CA9</x:v>
+      </x:c>
+      <x:c r="D25" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B26" s="1" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="C26" s="1" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="D26" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A26" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B26" s="1" t="str">
+        <x:v>chk6</x:v>
+      </x:c>
+      <x:c r="C26" s="1" t="str">
+        <x:v>CHK6</x:v>
+      </x:c>
+      <x:c r="D26" s="1" t="str">
+        <x:v>r5</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B27" s="1" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="C27" s="1" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="D27" s="1" t="s">
-        <x:v>18</x:v>
+      <x:c r="A27" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B27" s="1" t="str">
+        <x:v>cks1</x:v>
+      </x:c>
+      <x:c r="C27" s="1" t="str">
+        <x:v>CKS1</x:v>
+      </x:c>
+      <x:c r="D27" s="1" t="str">
+        <x:v>r8</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B28" s="1" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="C28" s="1" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="D28" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A28" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B28" s="1" t="str">
+        <x:v>cph2</x:v>
+      </x:c>
+      <x:c r="C28" s="1" t="str">
+        <x:v>CPH2</x:v>
+      </x:c>
+      <x:c r="D28" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B29" s="1" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="C29" s="1" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D29" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A29" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B29" s="1" t="str">
+        <x:v>cuk7</x:v>
+      </x:c>
+      <x:c r="C29" s="1" t="str">
+        <x:v>CUK7</x:v>
+      </x:c>
+      <x:c r="D29" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B30" s="1" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="C30" s="1" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="D30" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A30" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B30" s="1" t="str">
+        <x:v>kcg4</x:v>
+      </x:c>
+      <x:c r="C30" s="1" t="str">
+        <x:v>KCG4</x:v>
+      </x:c>
+      <x:c r="D30" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B31" s="1" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="C31" s="1" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="D31" s="1" t="s">
-        <x:v>14</x:v>
+      <x:c r="A31" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B31" s="1" t="str">
+        <x:v>kcm1</x:v>
+      </x:c>
+      <x:c r="C31" s="1" t="str">
+        <x:v>KCM1</x:v>
+      </x:c>
+      <x:c r="D31" s="1" t="str">
+        <x:v>r6</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B32" s="1" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="C32" s="1" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="D32" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A32" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B32" s="1" t="str">
+        <x:v>kdl1</x:v>
+      </x:c>
+      <x:c r="C32" s="1" t="str">
+        <x:v>KDL1</x:v>
+      </x:c>
+      <x:c r="D32" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B33" s="1" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="C33" s="1" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="D33" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A33" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B33" s="1" t="str">
+        <x:v>kht3</x:v>
+      </x:c>
+      <x:c r="C33" s="1" t="str">
+        <x:v>KHT3</x:v>
+      </x:c>
+      <x:c r="D33" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B34" s="1" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C34" s="1" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="D34" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A34" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B34" s="1" t="str">
+        <x:v>kkg3</x:v>
+      </x:c>
+      <x:c r="C34" s="1" t="str">
+        <x:v>KKG3</x:v>
+      </x:c>
+      <x:c r="D34" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B35" s="1" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="C35" s="1" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="D35" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A35" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B35" s="1" t="str">
+        <x:v>tpg2</x:v>
+      </x:c>
+      <x:c r="C35" s="1" t="str">
+        <x:v>TPG2</x:v>
+      </x:c>
+      <x:c r="D35" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B36" s="1" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="C36" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D36" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A36" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B36" s="1" t="str">
+        <x:v>kps7</x:v>
+      </x:c>
+      <x:c r="C36" s="1" t="str">
+        <x:v>KPS7</x:v>
+      </x:c>
+      <x:c r="D36" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B37" s="1" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="C37" s="1" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="D37" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A37" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B37" s="1" t="str">
+        <x:v>kpt2</x:v>
+      </x:c>
+      <x:c r="C37" s="1" t="str">
+        <x:v>KPT2</x:v>
+      </x:c>
+      <x:c r="D37" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B38" s="1" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="C38" s="1" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="D38" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A38" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B38" s="1" t="str">
+        <x:v>krg7</x:v>
+      </x:c>
+      <x:c r="C38" s="1" t="str">
+        <x:v>KRG7</x:v>
+      </x:c>
+      <x:c r="D38" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B39" s="1" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="C39" s="1" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="D39" s="1" t="s">
-        <x:v>16</x:v>
+      <x:c r="A39" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B39" s="1" t="str">
+        <x:v>krt1</x:v>
+      </x:c>
+      <x:c r="C39" s="1" t="str">
+        <x:v>KRT1</x:v>
+      </x:c>
+      <x:c r="D39" s="1" t="str">
+        <x:v>r7</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B40" s="1" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="C40" s="1" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="D40" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A40" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B40" s="1" t="str">
+        <x:v>krv5</x:v>
+      </x:c>
+      <x:c r="C40" s="1" t="str">
+        <x:v>KRV5</x:v>
+      </x:c>
+      <x:c r="D40" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B41" s="1" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="C41" s="1" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="D41" s="1" t="s">
-        <x:v>16</x:v>
+      <x:c r="A41" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B41" s="1" t="str">
+        <x:v>ksa5</x:v>
+      </x:c>
+      <x:c r="C41" s="1" t="str">
+        <x:v>KSA5</x:v>
+      </x:c>
+      <x:c r="D41" s="1" t="str">
+        <x:v>r7</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B42" s="1" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="C42" s="1" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="D42" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A42" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B42" s="1" t="str">
+        <x:v>ksm1</x:v>
+      </x:c>
+      <x:c r="C42" s="1" t="str">
+        <x:v>KSM1</x:v>
+      </x:c>
+      <x:c r="D42" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B43" s="1" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="C43" s="1" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="D43" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A43" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B43" s="1" t="str">
+        <x:v>ksp3</x:v>
+      </x:c>
+      <x:c r="C43" s="1" t="str">
+        <x:v>KSP3</x:v>
+      </x:c>
+      <x:c r="D43" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B44" s="1" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="C44" s="1" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="D44" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A44" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B44" s="1" t="str">
+        <x:v>ksv5</x:v>
+      </x:c>
+      <x:c r="C44" s="1" t="str">
+        <x:v>KSV5</x:v>
+      </x:c>
+      <x:c r="D44" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B45" s="1" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="C45" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D45" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A45" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B45" s="1" t="str">
+        <x:v>ktb1</x:v>
+      </x:c>
+      <x:c r="C45" s="1" t="str">
+        <x:v>KTB1</x:v>
+      </x:c>
+      <x:c r="D45" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B46" s="1" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="C46" s="1" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D46" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A46" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B46" s="1" t="str">
+        <x:v>kth2</x:v>
+      </x:c>
+      <x:c r="C46" s="1" t="str">
+        <x:v>KTH2</x:v>
+      </x:c>
+      <x:c r="D46" s="1" t="str">
+        <x:v>r5</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B47" s="1" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="C47" s="1" t="s">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="D47" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A47" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B47" s="1" t="str">
+        <x:v>ktl6</x:v>
+      </x:c>
+      <x:c r="C47" s="1" t="str">
+        <x:v>KTL6</x:v>
+      </x:c>
+      <x:c r="D47" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B48" s="1" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="C48" s="1" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="D48" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A48" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B48" s="1" t="str">
+        <x:v>ktm8</x:v>
+      </x:c>
+      <x:c r="C48" s="1" t="str">
+        <x:v>KTM8</x:v>
+      </x:c>
+      <x:c r="D48" s="1" t="str">
+        <x:v>r5</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B49" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="C49" s="1" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="D49" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A49" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B49" s="1" t="str">
+        <x:v>ktr4</x:v>
+      </x:c>
+      <x:c r="C49" s="1" t="str">
+        <x:v>KTR4</x:v>
+      </x:c>
+      <x:c r="D49" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B50" s="1" t="s">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="C50" s="1" t="s">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="D50" s="1" t="s">
-        <x:v>16</x:v>
+      <x:c r="A50" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B50" s="1" t="str">
+        <x:v>mdk2</x:v>
+      </x:c>
+      <x:c r="C50" s="1" t="str">
+        <x:v>MDK2</x:v>
+      </x:c>
+      <x:c r="D50" s="1" t="str">
+        <x:v>r7</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B51" s="1" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="C51" s="1" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="D51" s="1" t="s">
-        <x:v>14</x:v>
+      <x:c r="A51" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B51" s="1" t="str">
+        <x:v>mmt3</x:v>
+      </x:c>
+      <x:c r="C51" s="1" t="str">
+        <x:v>MMT3</x:v>
+      </x:c>
+      <x:c r="D51" s="1" t="str">
+        <x:v>r6</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B52" s="1" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="C52" s="1" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="D52" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A52" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B52" s="1" t="str">
+        <x:v>mrs5</x:v>
+      </x:c>
+      <x:c r="C52" s="1" t="str">
+        <x:v>MRS5</x:v>
+      </x:c>
+      <x:c r="D52" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B53" s="1" t="s">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="C53" s="1" t="s">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="D53" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A53" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B53" s="1" t="str">
+        <x:v>pkb4</x:v>
+      </x:c>
+      <x:c r="C53" s="1" t="str">
+        <x:v>PKB4</x:v>
+      </x:c>
+      <x:c r="D53" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B54" s="1" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="C54" s="1" t="s">
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="D54" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A54" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B54" s="1" t="str">
+        <x:v>pln4</x:v>
+      </x:c>
+      <x:c r="C54" s="1" t="str">
+        <x:v>PLN4</x:v>
+      </x:c>
+      <x:c r="D54" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B55" s="1" t="s">
-        <x:v>111</x:v>
-      </x:c>
-      <x:c r="C55" s="1" t="s">
-        <x:v>112</x:v>
-      </x:c>
-      <x:c r="D55" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A55" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B55" s="1" t="str">
+        <x:v>pmr5</x:v>
+      </x:c>
+      <x:c r="C55" s="1" t="str">
+        <x:v>PMR5</x:v>
+      </x:c>
+      <x:c r="D55" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B56" s="1" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="C56" s="1" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="D56" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A56" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B56" s="1" t="str">
+        <x:v>pnp6</x:v>
+      </x:c>
+      <x:c r="C56" s="1" t="str">
+        <x:v>PNP6</x:v>
+      </x:c>
+      <x:c r="D56" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B57" s="1" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="C57" s="1" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="D57" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A57" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B57" s="1" t="str">
+        <x:v>ppr8</x:v>
+      </x:c>
+      <x:c r="C57" s="1" t="str">
+        <x:v>PPR8</x:v>
+      </x:c>
+      <x:c r="D57" s="1" t="str">
+        <x:v>r5</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B58" s="1" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="C58" s="1" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="D58" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A58" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B58" s="1" t="str">
+        <x:v>ppt3</x:v>
+      </x:c>
+      <x:c r="C58" s="1" t="str">
+        <x:v>PPT3</x:v>
+      </x:c>
+      <x:c r="D58" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B59" s="1" t="s">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="C59" s="1" t="s">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="D59" s="1" t="s">
-        <x:v>4</x:v>
+      <x:c r="A59" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B59" s="1" t="str">
+        <x:v>ptm6</x:v>
+      </x:c>
+      <x:c r="C59" s="1" t="str">
+        <x:v>PTM6</x:v>
+      </x:c>
+      <x:c r="D59" s="1" t="str">
+        <x:v>r1</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B60" s="1" t="s">
-        <x:v>121</x:v>
-      </x:c>
-      <x:c r="C60" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="D60" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A60" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B60" s="1" t="str">
+        <x:v>puk7</x:v>
+      </x:c>
+      <x:c r="C60" s="1" t="str">
+        <x:v>PUK7</x:v>
+      </x:c>
+      <x:c r="D60" s="1" t="str">
+        <x:v>r5</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B61" s="1" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="C61" s="1" t="s">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="D61" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A61" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B61" s="1" t="str">
+        <x:v>pus5</x:v>
+      </x:c>
+      <x:c r="C61" s="1" t="str">
+        <x:v>PUS5</x:v>
+      </x:c>
+      <x:c r="D61" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B62" s="1" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="C62" s="1" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="D62" s="1" t="s">
-        <x:v>18</x:v>
+      <x:c r="A62" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B62" s="1" t="str">
+        <x:v>pvh3</x:v>
+      </x:c>
+      <x:c r="C62" s="1" t="str">
+        <x:v>PVH3</x:v>
+      </x:c>
+      <x:c r="D62" s="1" t="str">
+        <x:v>r8</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B63" s="1" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="C63" s="1" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="D63" s="1" t="s">
-        <x:v>16</x:v>
+      <x:c r="A63" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B63" s="1" t="str">
+        <x:v>rtk4</x:v>
+      </x:c>
+      <x:c r="C63" s="1" t="str">
+        <x:v>RTK4</x:v>
+      </x:c>
+      <x:c r="D63" s="1" t="str">
+        <x:v>r7</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B64" s="1" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="C64" s="1" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="D64" s="1" t="s">
-        <x:v>18</x:v>
+      <x:c r="A64" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B64" s="1" t="str">
+        <x:v>smr5</x:v>
+      </x:c>
+      <x:c r="C64" s="1" t="str">
+        <x:v>SMR5</x:v>
+      </x:c>
+      <x:c r="D64" s="1" t="str">
+        <x:v>r8</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B65" s="1" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="C65" s="1" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="D65" s="1" t="s">
-        <x:v>16</x:v>
+      <x:c r="A65" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B65" s="1" t="str">
+        <x:v>snl6</x:v>
+      </x:c>
+      <x:c r="C65" s="1" t="str">
+        <x:v>SNL6</x:v>
+      </x:c>
+      <x:c r="D65" s="1" t="str">
+        <x:v>r7</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B66" s="1" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="C66" s="1" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D66" s="1" t="s">
-        <x:v>8</x:v>
+      <x:c r="A66" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B66" s="1" t="str">
+        <x:v>sra5</x:v>
+      </x:c>
+      <x:c r="C66" s="1" t="str">
+        <x:v>SRA5</x:v>
+      </x:c>
+      <x:c r="D66" s="1" t="str">
+        <x:v>r3</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B67" s="1" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="C67" s="1" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D67" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A67" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B67" s="1" t="str">
+        <x:v>srp1</x:v>
+      </x:c>
+      <x:c r="C67" s="1" t="str">
+        <x:v>SRP1</x:v>
+      </x:c>
+      <x:c r="D67" s="1" t="str">
+        <x:v>r5</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B68" s="1" t="s">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="C68" s="1" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="D68" s="1" t="s">
-        <x:v>16</x:v>
+      <x:c r="A68" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B68" s="1" t="str">
+        <x:v>str3</x:v>
+      </x:c>
+      <x:c r="C68" s="1" t="str">
+        <x:v>STR3</x:v>
+      </x:c>
+      <x:c r="D68" s="1" t="str">
+        <x:v>r7</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B69" s="1" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="C69" s="1" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="D69" s="1" t="s">
-        <x:v>14</x:v>
+      <x:c r="A69" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B69" s="1" t="str">
+        <x:v>stt4</x:v>
+      </x:c>
+      <x:c r="C69" s="1" t="str">
+        <x:v>STT4</x:v>
+      </x:c>
+      <x:c r="D69" s="1" t="str">
+        <x:v>r6</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
-      <x:c r="A70" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B70" s="1" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="C70" s="1" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="D70" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A70" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B70" s="1" t="str">
+        <x:v>sva7</x:v>
+      </x:c>
+      <x:c r="C70" s="1" t="str">
+        <x:v>SVA7</x:v>
+      </x:c>
+      <x:c r="D70" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
-      <x:c r="A71" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B71" s="1" t="s">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="C71" s="1" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="D71" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A71" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B71" s="1" t="str">
+        <x:v>svr4</x:v>
+      </x:c>
+      <x:c r="C71" s="1" t="str">
+        <x:v>SVR4</x:v>
+      </x:c>
+      <x:c r="D71" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B72" s="1" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="C72" s="1" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="D72" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="A72" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B72" s="1" t="str">
+        <x:v>tak2</x:v>
+      </x:c>
+      <x:c r="C72" s="1" t="str">
+        <x:v>TAK2</x:v>
+      </x:c>
+      <x:c r="D72" s="1" t="str">
+        <x:v>r2</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B73" s="1" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C73" s="1" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D73" s="1" t="s">
-        <x:v>14</x:v>
+      <x:c r="A73" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B73" s="1" t="str">
+        <x:v>tkm2</x:v>
+      </x:c>
+      <x:c r="C73" s="1" t="str">
+        <x:v>TKM2</x:v>
+      </x:c>
+      <x:c r="D73" s="1" t="str">
+        <x:v>r6</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
-      <x:c r="A74" s="1" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B74" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="C74" s="1" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D74" s="1" t="s">
-        <x:v>10</x:v>
+      <x:c r="A74" s="1" t="str">
+        <x:v>dealer</x:v>
+      </x:c>
+      <x:c r="B74" s="1" t="str">
+        <x:v>vvg1</x:v>
+      </x:c>
+      <x:c r="C74" s="1" t="str">
+        <x:v>VVG1</x:v>
+      </x:c>
+      <x:c r="D74" s="1" t="str">
+        <x:v>r4</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="5.75" customHeight="1">
-      <x:c r="A75" s="1" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B75" s="1" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C75" s="1" t="s">
-        <x:v>153</x:v>
+      <x:c r="A75" s="1" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B75" s="1" t="str">
+        <x:v>wholesale</x:v>
+      </x:c>
+      <x:c r="C75" s="1" t="str">
+        <x:v>Wholesale</x:v>
       </x:c>
       <x:c r="D75" s="1"/>
     </x:row>
     <x:row r="76" ht="5.75" customHeight="1">
-      <x:c r="A76" s="1" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B76" s="1" t="s">
-        <x:v>154</x:v>
-      </x:c>
-      <x:c r="C76" s="1" t="s">
-        <x:v>155</x:v>
+      <x:c r="A76" s="1" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B76" s="1" t="str">
+        <x:v>drink_shop</x:v>
+      </x:c>
+      <x:c r="C76" s="1" t="str">
+        <x:v>Drink Shop</x:v>
       </x:c>
       <x:c r="D76" s="1"/>
     </x:row>
     <x:row r="77" ht="5.75" customHeight="1">
-      <x:c r="A77" s="1" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B77" s="1" t="s">
-        <x:v>156</x:v>
-      </x:c>
-      <x:c r="C77" s="1" t="s">
-        <x:v>157</x:v>
+      <x:c r="A77" s="1" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B77" s="1" t="str">
+        <x:v>wet_market</x:v>
+      </x:c>
+      <x:c r="C77" s="1" t="str">
+        <x:v>Wet Market</x:v>
       </x:c>
       <x:c r="D77" s="1"/>
     </x:row>
     <x:row r="78" ht="5.75" customHeight="1">
-      <x:c r="A78" s="1" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B78" s="1" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="C78" s="1" t="s">
-        <x:v>159</x:v>
+      <x:c r="A78" s="1" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B78" s="1" t="str">
+        <x:v>trolley</x:v>
+      </x:c>
+      <x:c r="C78" s="1" t="str">
+        <x:v>Trolley</x:v>
       </x:c>
       <x:c r="D78" s="1"/>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="1" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="B79" s="1" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="C79" s="1" t="s">
-        <x:v>162</x:v>
+      <x:c r="A79" s="1" t="str">
+        <x:v>yes_no</x:v>
+      </x:c>
+      <x:c r="B79" s="1" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="C79" s="1" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="D79" s="1"/>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="1" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="B80" s="1" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="C80" s="1" t="s">
-        <x:v>164</x:v>
+      <x:c r="A80" s="1" t="str">
+        <x:v>yes_no</x:v>
+      </x:c>
+      <x:c r="B80" s="1" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="C80" s="1" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="D80" s="1"/>
     </x:row>
     <x:row r="81" ht="5.75" customHeight="1">
-      <x:c r="A81" s="1" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="B81" s="1" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="C81" s="1" t="s">
-        <x:v>167</x:v>
+      <x:c r="A81" s="1" t="str">
+        <x:v>stock_status</x:v>
+      </x:c>
+      <x:c r="B81" s="1" t="str">
+        <x:v>full</x:v>
+      </x:c>
+      <x:c r="C81" s="1" t="str">
+        <x:v>គ្រប់</x:v>
       </x:c>
       <x:c r="D81" s="1"/>
     </x:row>
     <x:row r="82" ht="5.75" customHeight="1">
-      <x:c r="A82" s="1" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="B82" s="1" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="C82" s="1" t="s">
-        <x:v>169</x:v>
+      <x:c r="A82" s="1" t="str">
+        <x:v>stock_status</x:v>
+      </x:c>
+      <x:c r="B82" s="1" t="str">
+        <x:v>low</x:v>
+      </x:c>
+      <x:c r="C82" s="1" t="str">
+        <x:v>ខ្វះ</x:v>
       </x:c>
       <x:c r="D82" s="1"/>
     </x:row>
     <x:row r="83" ht="5.75" customHeight="1">
-      <x:c r="A83" s="1" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="B83" s="1" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="C83" s="1" t="s">
-        <x:v>171</x:v>
+      <x:c r="A83" s="1" t="str">
+        <x:v>stock_status</x:v>
+      </x:c>
+      <x:c r="B83" s="1" t="str">
+        <x:v>no_stock</x:v>
+      </x:c>
+      <x:c r="C83" s="1" t="str">
+        <x:v>ដាច់ស្តុក</x:v>
       </x:c>
       <x:c r="D83" s="1"/>
     </x:row>
     <x:row r="84" ht="5.75" customHeight="1">
-      <x:c r="A84" s="1" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="B84" s="1" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="C84" s="1" t="s">
-        <x:v>174</x:v>
+      <x:c r="A84" s="1" t="str">
+        <x:v>movement_score</x:v>
+      </x:c>
+      <x:c r="B84" s="1" t="str">
+        <x:v>no_sale</x:v>
+      </x:c>
+      <x:c r="C84" s="1" t="str">
+        <x:v>អត់មានលក់</x:v>
       </x:c>
       <x:c r="D84" s="1"/>
     </x:row>
     <x:row r="85" ht="5.75" customHeight="1">
-      <x:c r="A85" s="1" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="B85" s="1" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="C85" s="1" t="s">
-        <x:v>176</x:v>
+      <x:c r="A85" s="1" t="str">
+        <x:v>movement_score</x:v>
+      </x:c>
+      <x:c r="B85" s="1" t="str">
+        <x:v>sale</x:v>
+      </x:c>
+      <x:c r="C85" s="1" t="str">
+        <x:v>មានលក់</x:v>
       </x:c>
       <x:c r="D85" s="1"/>
     </x:row>
     <x:row r="86" ht="5.75" customHeight="1">
-      <x:c r="A86" s="1" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="B86" s="1" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="C86" s="1" t="s">
-        <x:v>178</x:v>
+      <x:c r="A86" s="1" t="str">
+        <x:v>movement_score</x:v>
+      </x:c>
+      <x:c r="B86" s="1" t="str">
+        <x:v>fast_sale</x:v>
+      </x:c>
+      <x:c r="C86" s="1" t="str">
+        <x:v>លក់ដាច់</x:v>
       </x:c>
       <x:c r="D86" s="1"/>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="B87" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="C87" t="s">
-        <x:v>181</x:v>
-      </x:c>
+      <x:c r="A87" t="str">
+        <x:v>ring_pull_in_outlet_choices</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>cbl_ncp_6_can</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>CBL NCP 6 Can</x:v>
+      </x:c>
+      <x:c r="D87"/>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="B88" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="C88" t="s">
-        <x:v>183</x:v>
-      </x:c>
+      <x:c r="A88" t="str">
+        <x:v>ring_pull_in_outlet_choices</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>cbl_ncp_5_usd</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>CBL NCP 5 USD</x:v>
+      </x:c>
+      <x:c r="D88"/>
     </x:row>
     <x:row r="89">
-      <x:c r="A89" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B89" t="s">
-        <x:v>184</x:v>
-      </x:c>
-      <x:c r="C89" t="s">
-        <x:v>185</x:v>
-      </x:c>
+      <x:c r="A89" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>local_eat</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>Local Eat</x:v>
+      </x:c>
+      <x:c r="D89"/>
     </x:row>
     <x:row r="90">
-      <x:c r="A90" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B90" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C90" t="s">
-        <x:v>187</x:v>
-      </x:c>
+      <x:c r="A90" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>coffee_bakery</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>Coffee,Bakery</x:v>
+      </x:c>
+      <x:c r="D90"/>
     </x:row>
     <x:row r="91">
-      <x:c r="A91" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B91" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="C91" t="s">
-        <x:v>189</x:v>
-      </x:c>
+      <x:c r="A91" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>canteen</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>Canteen</x:v>
+      </x:c>
+      <x:c r="D91"/>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B92" t="s">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="C92" t="s">
-        <x:v>191</x:v>
-      </x:c>
+      <x:c r="A92" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>sport_club</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>Sport Club</x:v>
+      </x:c>
+      <x:c r="D92"/>
     </x:row>
     <x:row r="93">
-      <x:c r="A93" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="B93" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="C93" t="s">
-        <x:v>193</x:v>
-      </x:c>
+      <x:c r="A93" t="str">
+        <x:v>outlet_type</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>motor_shop</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>Motor Shop</x:v>
+      </x:c>
+      <x:c r="D93"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>summary_report_type</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>channel_specialist</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>CHANNEL SPECIALIST</x:v>
+      </x:c>
+      <x:c r="D94"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14677,18 +14141,18 @@
   <x:sheetData>
     <x:row r="1" ht="5.75" customHeight="1">
       <x:c r="A1" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>195</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="17.149999618530273" customHeight="1">
       <x:c r="A2" s="1" t="s">
-        <x:v>196</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>197</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14798,10 +14262,10 @@
         <x:v>8. Outlet comments and final summary</x:v>
       </x:c>
       <x:c r="B9" s="1" t="str">
-        <x:v>Every outlet may enter Key Issues/Suggestions; only latest row with a summary-marker Outlet Name is selected</x:v>
+        <x:v>Summary-marker row: blank template selector = GENERAL; CHANNEL SPECIALIST selector = Channel Specialist summary</x:v>
       </x:c>
       <x:c r="C9" s="1" t="str">
-        <x:v>Normal comments stored but ignored for final summary; marker row supplies 4 + 4 report points</x:v>
+        <x:v>General and Channel Specialist summaries are selected independently</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25.75" customHeight="1">
@@ -15908,13 +15372,13 @@
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="C63" s="1" t="str">
-        <x:v>Key Issues</x:v>
+        <x:v>Summary Template</x:v>
       </x:c>
       <x:c r="D63" s="1" t="str">
-        <x:v>key_issues_detail</x:v>
+        <x:v>final_summary_report_type</x:v>
       </x:c>
       <x:c r="E63" s="1" t="str">
-        <x:v>Latest accepted-keyword submission only; up to 4 points.</x:v>
+        <x:v>Blank = GENERAL; channel_specialist = CHANNEL SPECIALIST</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -15925,12 +15389,29 @@
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="C64" s="1" t="str">
+        <x:v>Key Issues</x:v>
+      </x:c>
+      <x:c r="D64" s="1" t="str">
+        <x:v>key_issues_detail</x:v>
+      </x:c>
+      <x:c r="E64" s="1" t="str">
+        <x:v>Latest accepted-keyword submission only; up to 4 points.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>Summary</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
         <x:v>Initiative Idea / Suggestion</x:v>
       </x:c>
-      <x:c r="D64" s="1" t="str">
+      <x:c r="D65" t="str">
         <x:v>initiative_idea_suggestion</x:v>
       </x:c>
-      <x:c r="E64" s="1" t="str">
+      <x:c r="E65" t="str">
         <x:v>Latest accepted-keyword submission only; up to 4 points.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Fix Khmer PNG and route summaries by report template
</commit_message>
<xml_diff>
--- a/templates/KB_Market_Improvement_XLSForm.xlsx
+++ b/templates/KB_Market_Improvement_XLSForm.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R6575acf8648e4da3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R9939f5cf871a43c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rd8e5222235b1401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="Rc19bfc70e32e402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="R7414df225b0e4d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Recc9d1d7dd774762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rce1793ab7c094f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R7385a5c67aca459c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="R0b02933b9938481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="R397e2b0247384136"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2919,12 +2919,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">summary_instruction</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FINAL KEY ISSUES &amp; INITIATIVE IDEA / SUGGESTION</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Set Outlet Name to an accepted summary keyword. Leave Summary Template blank for GENERAL, or select CHANNEL SPECIALIST for the Channel Specialist report. Then enter up to 4 Key Issues and 4 Initiative/Suggestion points.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">select_one summary_report_type</x:t>
@@ -16773,14 +16767,14 @@
       <x:c r="B488" s="1" t="s">
         <x:v>968</x:v>
       </x:c>
-      <x:c r="C488" s="1" t="s">
-        <x:v>969</x:v>
+      <x:c r="C488" s="1" t="str">
+        <x:v>សេចក្តីសង្ខេបចុងក្រោយ / FINAL KEY ISSUES &amp; INITIATIVE IDEA / SUGGESTION</x:v>
       </x:c>
       <x:c r="D488" s="1" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E488" s="1" t="s">
-        <x:v>970</x:v>
+      <x:c r="E488" s="1" t="str">
+        <x:v>សូមបញ្ចូល Outlet Name ជាពាក្យសង្ខេបដែលបានកំណត់។ សម្រាប់ GT / GENERAL សូមទុក Summary Template ឱ្យទទេ។ សម្រាប់ CHANNEL SPECIALIST សូមជ្រើសរើស CHANNEL SPECIALIST។ បន្ទាប់មកបញ្ចូល Key Issues និង Initiative / Suggestion បានរហូតដល់ 4 ចំណុច។</x:v>
       </x:c>
       <x:c r="F488" s="1"/>
       <x:c r="G488" s="1"/>
@@ -16791,10 +16785,10 @@
     </x:row>
     <x:row r="489" ht="54" customHeight="1">
       <x:c r="A489" s="1" t="s">
-        <x:v>971</x:v>
+        <x:v>969</x:v>
       </x:c>
       <x:c r="B489" s="1" t="s">
-        <x:v>972</x:v>
+        <x:v>970</x:v>
       </x:c>
       <x:c r="C489" s="1" t="str">
         <x:v>&lt;span style="color:red"&gt;Summary Template / ប្រភេទរបាយការណ៍&lt;/span&gt;</x:v>
@@ -16803,14 +16797,14 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E489" s="1" t="str">
-        <x:v>ប្រសិនបើ Report របស់បងៗជាប្រភេទ CHANNEL SPECIALIST សូមជ្រើសរើស CHANNEL SPECIALIST។ បើ Report របស់បងៗជាប្រភេទ GT សូមកុំជ្រើសរើស។</x:v>
+        <x:v>ប្រសិនបើ Report របស់បងៗជាប្រភេទ CHANNEL SPECIALIST សូមជ្រើសរើស CHANNEL SPECIALIST។ បើ Report របស់បងៗជាប្រភេទ GT / GENERAL សូមទុកចន្លោះនេះឱ្យទទេ។</x:v>
       </x:c>
       <x:c r="F489" s="1" t="s">
         <x:v>20</x:v>
       </x:c>
       <x:c r="G489" s="1"/>
       <x:c r="H489" s="1" t="s">
-        <x:v>973</x:v>
+        <x:v>971</x:v>
       </x:c>
       <x:c r="I489" s="1"/>
       <x:c r="J489" s="1"/>
@@ -16821,19 +16815,19 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B490" s="1" t="s">
+        <x:v>972</x:v>
+      </x:c>
+      <x:c r="C490" s="1" t="s">
+        <x:v>973</x:v>
+      </x:c>
+      <x:c r="D490" s="1" t="s">
+        <x:v>971</x:v>
+      </x:c>
+      <x:c r="E490" s="1" t="s">
         <x:v>974</x:v>
       </x:c>
-      <x:c r="C490" s="1" t="s">
+      <x:c r="F490" s="1" t="s">
         <x:v>975</x:v>
-      </x:c>
-      <x:c r="D490" s="1" t="s">
-        <x:v>973</x:v>
-      </x:c>
-      <x:c r="E490" s="1" t="s">
-        <x:v>976</x:v>
-      </x:c>
-      <x:c r="F490" s="1" t="s">
-        <x:v>977</x:v>
       </x:c>
       <x:c r="G490" s="1"/>
       <x:c r="H490" s="1"/>
@@ -16846,19 +16840,19 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B491" s="1" t="s">
+        <x:v>976</x:v>
+      </x:c>
+      <x:c r="C491" s="1" t="s">
+        <x:v>977</x:v>
+      </x:c>
+      <x:c r="D491" s="1" t="s">
+        <x:v>971</x:v>
+      </x:c>
+      <x:c r="E491" s="1" t="s">
         <x:v>978</x:v>
       </x:c>
-      <x:c r="C491" s="1" t="s">
-        <x:v>979</x:v>
-      </x:c>
-      <x:c r="D491" s="1" t="s">
-        <x:v>973</x:v>
-      </x:c>
-      <x:c r="E491" s="1" t="s">
-        <x:v>980</x:v>
-      </x:c>
       <x:c r="F491" s="1" t="s">
-        <x:v>977</x:v>
+        <x:v>975</x:v>
       </x:c>
       <x:c r="G491" s="1"/>
       <x:c r="H491" s="1"/>
@@ -16885,7 +16879,7 @@
   <x:sheetData>
     <x:row r="1" ht="3.9000000953674316" customHeight="1">
       <x:c r="A1" s="2" t="s">
-        <x:v>981</x:v>
+        <x:v>979</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
         <x:v>1</x:v>
@@ -16902,10 +16896,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>983</x:v>
+        <x:v>981</x:v>
       </x:c>
       <x:c r="D2" s="1"/>
     </x:row>
@@ -16914,10 +16908,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
-        <x:v>985</x:v>
+        <x:v>983</x:v>
       </x:c>
       <x:c r="D3" s="1"/>
     </x:row>
@@ -16926,10 +16920,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B4" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>987</x:v>
+        <x:v>985</x:v>
       </x:c>
       <x:c r="D4" s="1"/>
     </x:row>
@@ -16938,10 +16932,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B5" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
-        <x:v>989</x:v>
+        <x:v>987</x:v>
       </x:c>
       <x:c r="D5" s="1"/>
     </x:row>
@@ -16950,10 +16944,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>991</x:v>
+        <x:v>989</x:v>
       </x:c>
       <x:c r="D6" s="1"/>
     </x:row>
@@ -16962,10 +16956,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>992</x:v>
+        <x:v>990</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>993</x:v>
+        <x:v>991</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
     </x:row>
@@ -16974,10 +16968,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>995</x:v>
+        <x:v>993</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
     </x:row>
@@ -16986,10 +16980,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>996</x:v>
+        <x:v>994</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>997</x:v>
+        <x:v>995</x:v>
       </x:c>
       <x:c r="D9" s="1"/>
     </x:row>
@@ -16998,13 +16992,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>998</x:v>
+        <x:v>996</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>999</x:v>
+        <x:v>997</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>996</x:v>
+        <x:v>994</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -17012,13 +17006,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>1000</x:v>
+        <x:v>998</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>1001</x:v>
+        <x:v>999</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -17026,13 +17020,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>1002</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>1003</x:v>
+        <x:v>1001</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -17040,13 +17034,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>1004</x:v>
+        <x:v>1002</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>1005</x:v>
+        <x:v>1003</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -17054,13 +17048,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>1006</x:v>
+        <x:v>1004</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>1007</x:v>
+        <x:v>1005</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -17068,13 +17062,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>1008</x:v>
+        <x:v>1006</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>1009</x:v>
+        <x:v>1007</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>992</x:v>
+        <x:v>990</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -17082,13 +17076,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
-        <x:v>1010</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>1011</x:v>
+        <x:v>1009</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -17096,13 +17090,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>1012</x:v>
+        <x:v>1010</x:v>
       </x:c>
       <x:c r="C17" s="1" t="s">
-        <x:v>1013</x:v>
+        <x:v>1011</x:v>
       </x:c>
       <x:c r="D17" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -17110,13 +17104,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>1014</x:v>
+        <x:v>1012</x:v>
       </x:c>
       <x:c r="C18" s="1" t="s">
-        <x:v>1015</x:v>
+        <x:v>1013</x:v>
       </x:c>
       <x:c r="D18" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -17124,13 +17118,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B19" s="1" t="s">
-        <x:v>1016</x:v>
+        <x:v>1014</x:v>
       </x:c>
       <x:c r="C19" s="1" t="s">
-        <x:v>1017</x:v>
+        <x:v>1015</x:v>
       </x:c>
       <x:c r="D19" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -17138,13 +17132,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
-        <x:v>1018</x:v>
+        <x:v>1016</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
-        <x:v>1019</x:v>
+        <x:v>1017</x:v>
       </x:c>
       <x:c r="D20" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -17152,13 +17146,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
-        <x:v>1020</x:v>
+        <x:v>1018</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
-        <x:v>1021</x:v>
+        <x:v>1019</x:v>
       </x:c>
       <x:c r="D21" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -17166,13 +17160,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>1022</x:v>
+        <x:v>1020</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>1023</x:v>
+        <x:v>1021</x:v>
       </x:c>
       <x:c r="D22" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -17180,13 +17174,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>1024</x:v>
+        <x:v>1022</x:v>
       </x:c>
       <x:c r="C23" s="1" t="s">
-        <x:v>1025</x:v>
+        <x:v>1023</x:v>
       </x:c>
       <x:c r="D23" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -17194,13 +17188,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>1026</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="C24" s="1" t="s">
-        <x:v>1027</x:v>
+        <x:v>1025</x:v>
       </x:c>
       <x:c r="D24" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -17208,13 +17202,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
-        <x:v>1028</x:v>
+        <x:v>1026</x:v>
       </x:c>
       <x:c r="C25" s="1" t="s">
-        <x:v>1029</x:v>
+        <x:v>1027</x:v>
       </x:c>
       <x:c r="D25" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -17222,13 +17216,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
-        <x:v>1030</x:v>
+        <x:v>1028</x:v>
       </x:c>
       <x:c r="C26" s="1" t="s">
-        <x:v>1031</x:v>
+        <x:v>1029</x:v>
       </x:c>
       <x:c r="D26" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -17236,13 +17230,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
-        <x:v>1032</x:v>
+        <x:v>1030</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
-        <x:v>1033</x:v>
+        <x:v>1031</x:v>
       </x:c>
       <x:c r="D27" s="1" t="s">
-        <x:v>996</x:v>
+        <x:v>994</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -17250,13 +17244,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B28" s="1" t="s">
-        <x:v>1034</x:v>
+        <x:v>1032</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
-        <x:v>1035</x:v>
+        <x:v>1033</x:v>
       </x:c>
       <x:c r="D28" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -17264,13 +17258,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
-        <x:v>1036</x:v>
+        <x:v>1034</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
-        <x:v>1037</x:v>
+        <x:v>1035</x:v>
       </x:c>
       <x:c r="D29" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -17278,13 +17272,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
-        <x:v>1038</x:v>
+        <x:v>1036</x:v>
       </x:c>
       <x:c r="C30" s="1" t="s">
-        <x:v>1039</x:v>
+        <x:v>1037</x:v>
       </x:c>
       <x:c r="D30" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -17292,13 +17286,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
-        <x:v>1040</x:v>
+        <x:v>1038</x:v>
       </x:c>
       <x:c r="C31" s="1" t="s">
-        <x:v>1041</x:v>
+        <x:v>1039</x:v>
       </x:c>
       <x:c r="D31" s="1" t="s">
-        <x:v>992</x:v>
+        <x:v>990</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -17306,13 +17300,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B32" s="1" t="s">
-        <x:v>1042</x:v>
+        <x:v>1040</x:v>
       </x:c>
       <x:c r="C32" s="1" t="s">
-        <x:v>1043</x:v>
+        <x:v>1041</x:v>
       </x:c>
       <x:c r="D32" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -17320,13 +17314,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B33" s="1" t="s">
-        <x:v>1044</x:v>
+        <x:v>1042</x:v>
       </x:c>
       <x:c r="C33" s="1" t="s">
-        <x:v>1045</x:v>
+        <x:v>1043</x:v>
       </x:c>
       <x:c r="D33" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -17334,13 +17328,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B34" s="1" t="s">
-        <x:v>1046</x:v>
+        <x:v>1044</x:v>
       </x:c>
       <x:c r="C34" s="1" t="s">
-        <x:v>1047</x:v>
+        <x:v>1045</x:v>
       </x:c>
       <x:c r="D34" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -17348,13 +17342,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B35" s="1" t="s">
-        <x:v>1048</x:v>
+        <x:v>1046</x:v>
       </x:c>
       <x:c r="C35" s="1" t="s">
-        <x:v>1049</x:v>
+        <x:v>1047</x:v>
       </x:c>
       <x:c r="D35" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -17362,13 +17356,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B36" s="1" t="s">
-        <x:v>1050</x:v>
+        <x:v>1048</x:v>
       </x:c>
       <x:c r="C36" s="1" t="s">
-        <x:v>1051</x:v>
+        <x:v>1049</x:v>
       </x:c>
       <x:c r="D36" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -17376,13 +17370,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
-        <x:v>1052</x:v>
+        <x:v>1050</x:v>
       </x:c>
       <x:c r="C37" s="1" t="s">
-        <x:v>1053</x:v>
+        <x:v>1051</x:v>
       </x:c>
       <x:c r="D37" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -17390,13 +17384,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>1054</x:v>
+        <x:v>1052</x:v>
       </x:c>
       <x:c r="C38" s="1" t="s">
-        <x:v>1055</x:v>
+        <x:v>1053</x:v>
       </x:c>
       <x:c r="D38" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -17404,13 +17398,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
-        <x:v>1056</x:v>
+        <x:v>1054</x:v>
       </x:c>
       <x:c r="C39" s="1" t="s">
-        <x:v>1057</x:v>
+        <x:v>1055</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -17418,13 +17412,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
-        <x:v>1058</x:v>
+        <x:v>1056</x:v>
       </x:c>
       <x:c r="C40" s="1" t="s">
-        <x:v>1059</x:v>
+        <x:v>1057</x:v>
       </x:c>
       <x:c r="D40" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -17432,13 +17426,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
-        <x:v>1060</x:v>
+        <x:v>1058</x:v>
       </x:c>
       <x:c r="C41" s="1" t="s">
-        <x:v>1061</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="D41" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -17446,13 +17440,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B42" s="1" t="s">
-        <x:v>1062</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="C42" s="1" t="s">
-        <x:v>1063</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="D42" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -17460,13 +17454,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B43" s="1" t="s">
-        <x:v>1064</x:v>
+        <x:v>1062</x:v>
       </x:c>
       <x:c r="C43" s="1" t="s">
-        <x:v>1065</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="D43" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -17474,13 +17468,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B44" s="1" t="s">
-        <x:v>1066</x:v>
+        <x:v>1064</x:v>
       </x:c>
       <x:c r="C44" s="1" t="s">
-        <x:v>1067</x:v>
+        <x:v>1065</x:v>
       </x:c>
       <x:c r="D44" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -17488,13 +17482,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B45" s="1" t="s">
-        <x:v>1068</x:v>
+        <x:v>1066</x:v>
       </x:c>
       <x:c r="C45" s="1" t="s">
-        <x:v>1069</x:v>
+        <x:v>1067</x:v>
       </x:c>
       <x:c r="D45" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -17502,13 +17496,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B46" s="1" t="s">
-        <x:v>1070</x:v>
+        <x:v>1068</x:v>
       </x:c>
       <x:c r="C46" s="1" t="s">
-        <x:v>1071</x:v>
+        <x:v>1069</x:v>
       </x:c>
       <x:c r="D46" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -17516,13 +17510,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B47" s="1" t="s">
-        <x:v>1072</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="C47" s="1" t="s">
-        <x:v>1073</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="D47" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -17530,13 +17524,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B48" s="1" t="s">
-        <x:v>1074</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="C48" s="1" t="s">
-        <x:v>1075</x:v>
+        <x:v>1073</x:v>
       </x:c>
       <x:c r="D48" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -17544,13 +17538,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B49" s="1" t="s">
-        <x:v>1076</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="C49" s="1" t="s">
-        <x:v>1077</x:v>
+        <x:v>1075</x:v>
       </x:c>
       <x:c r="D49" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -17558,13 +17552,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B50" s="1" t="s">
-        <x:v>1078</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="C50" s="1" t="s">
-        <x:v>1079</x:v>
+        <x:v>1077</x:v>
       </x:c>
       <x:c r="D50" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -17572,13 +17566,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B51" s="1" t="s">
-        <x:v>1080</x:v>
+        <x:v>1078</x:v>
       </x:c>
       <x:c r="C51" s="1" t="s">
-        <x:v>1081</x:v>
+        <x:v>1079</x:v>
       </x:c>
       <x:c r="D51" s="1" t="s">
-        <x:v>992</x:v>
+        <x:v>990</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -17586,13 +17580,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B52" s="1" t="s">
-        <x:v>1082</x:v>
+        <x:v>1080</x:v>
       </x:c>
       <x:c r="C52" s="1" t="s">
-        <x:v>1083</x:v>
+        <x:v>1081</x:v>
       </x:c>
       <x:c r="D52" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -17600,13 +17594,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B53" s="1" t="s">
-        <x:v>1084</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="C53" s="1" t="s">
-        <x:v>1085</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="D53" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -17614,13 +17608,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B54" s="1" t="s">
-        <x:v>1086</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="C54" s="1" t="s">
-        <x:v>1087</x:v>
+        <x:v>1085</x:v>
       </x:c>
       <x:c r="D54" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -17628,13 +17622,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B55" s="1" t="s">
-        <x:v>1088</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="C55" s="1" t="s">
-        <x:v>1089</x:v>
+        <x:v>1087</x:v>
       </x:c>
       <x:c r="D55" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -17642,13 +17636,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B56" s="1" t="s">
-        <x:v>1090</x:v>
+        <x:v>1088</x:v>
       </x:c>
       <x:c r="C56" s="1" t="s">
-        <x:v>1091</x:v>
+        <x:v>1089</x:v>
       </x:c>
       <x:c r="D56" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -17656,13 +17650,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B57" s="1" t="s">
-        <x:v>1092</x:v>
+        <x:v>1090</x:v>
       </x:c>
       <x:c r="C57" s="1" t="s">
-        <x:v>1093</x:v>
+        <x:v>1091</x:v>
       </x:c>
       <x:c r="D57" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -17670,13 +17664,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B58" s="1" t="s">
-        <x:v>1094</x:v>
+        <x:v>1092</x:v>
       </x:c>
       <x:c r="C58" s="1" t="s">
-        <x:v>1095</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="D58" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -17684,13 +17678,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B59" s="1" t="s">
-        <x:v>1096</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="C59" s="1" t="s">
-        <x:v>1097</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="D59" s="1" t="s">
-        <x:v>982</x:v>
+        <x:v>980</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -17698,13 +17692,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B60" s="1" t="s">
-        <x:v>1098</x:v>
+        <x:v>1096</x:v>
       </x:c>
       <x:c r="C60" s="1" t="s">
-        <x:v>1099</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="D60" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -17712,13 +17706,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B61" s="1" t="s">
-        <x:v>1100</x:v>
+        <x:v>1098</x:v>
       </x:c>
       <x:c r="C61" s="1" t="s">
-        <x:v>1101</x:v>
+        <x:v>1099</x:v>
       </x:c>
       <x:c r="D61" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -17726,13 +17720,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B62" s="1" t="s">
-        <x:v>1102</x:v>
+        <x:v>1100</x:v>
       </x:c>
       <x:c r="C62" s="1" t="s">
-        <x:v>1103</x:v>
+        <x:v>1101</x:v>
       </x:c>
       <x:c r="D62" s="1" t="s">
-        <x:v>996</x:v>
+        <x:v>994</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -17740,13 +17734,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B63" s="1" t="s">
-        <x:v>1104</x:v>
+        <x:v>1102</x:v>
       </x:c>
       <x:c r="C63" s="1" t="s">
-        <x:v>1105</x:v>
+        <x:v>1103</x:v>
       </x:c>
       <x:c r="D63" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -17754,13 +17748,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B64" s="1" t="s">
-        <x:v>1106</x:v>
+        <x:v>1104</x:v>
       </x:c>
       <x:c r="C64" s="1" t="s">
-        <x:v>1107</x:v>
+        <x:v>1105</x:v>
       </x:c>
       <x:c r="D64" s="1" t="s">
-        <x:v>996</x:v>
+        <x:v>994</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -17768,13 +17762,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B65" s="1" t="s">
-        <x:v>1108</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="C65" s="1" t="s">
-        <x:v>1109</x:v>
+        <x:v>1107</x:v>
       </x:c>
       <x:c r="D65" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -17782,13 +17776,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B66" s="1" t="s">
-        <x:v>1110</x:v>
+        <x:v>1108</x:v>
       </x:c>
       <x:c r="C66" s="1" t="s">
-        <x:v>1111</x:v>
+        <x:v>1109</x:v>
       </x:c>
       <x:c r="D66" s="1" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -17796,13 +17790,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B67" s="1" t="s">
-        <x:v>1112</x:v>
+        <x:v>1110</x:v>
       </x:c>
       <x:c r="C67" s="1" t="s">
-        <x:v>1113</x:v>
+        <x:v>1111</x:v>
       </x:c>
       <x:c r="D67" s="1" t="s">
-        <x:v>990</x:v>
+        <x:v>988</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -17810,13 +17804,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B68" s="1" t="s">
-        <x:v>1114</x:v>
+        <x:v>1112</x:v>
       </x:c>
       <x:c r="C68" s="1" t="s">
-        <x:v>1115</x:v>
+        <x:v>1113</x:v>
       </x:c>
       <x:c r="D68" s="1" t="s">
-        <x:v>994</x:v>
+        <x:v>992</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -17824,13 +17818,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B69" s="1" t="s">
-        <x:v>1116</x:v>
+        <x:v>1114</x:v>
       </x:c>
       <x:c r="C69" s="1" t="s">
-        <x:v>1117</x:v>
+        <x:v>1115</x:v>
       </x:c>
       <x:c r="D69" s="1" t="s">
-        <x:v>992</x:v>
+        <x:v>990</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -17838,13 +17832,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B70" s="1" t="s">
-        <x:v>1118</x:v>
+        <x:v>1116</x:v>
       </x:c>
       <x:c r="C70" s="1" t="s">
-        <x:v>1119</x:v>
+        <x:v>1117</x:v>
       </x:c>
       <x:c r="D70" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -17852,13 +17846,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B71" s="1" t="s">
-        <x:v>1120</x:v>
+        <x:v>1118</x:v>
       </x:c>
       <x:c r="C71" s="1" t="s">
-        <x:v>1121</x:v>
+        <x:v>1119</x:v>
       </x:c>
       <x:c r="D71" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -17866,13 +17860,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B72" s="1" t="s">
-        <x:v>1122</x:v>
+        <x:v>1120</x:v>
       </x:c>
       <x:c r="C72" s="1" t="s">
-        <x:v>1123</x:v>
+        <x:v>1121</x:v>
       </x:c>
       <x:c r="D72" s="1" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -17880,13 +17874,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B73" s="1" t="s">
-        <x:v>1124</x:v>
+        <x:v>1122</x:v>
       </x:c>
       <x:c r="C73" s="1" t="s">
-        <x:v>1125</x:v>
+        <x:v>1123</x:v>
       </x:c>
       <x:c r="D73" s="1" t="s">
-        <x:v>992</x:v>
+        <x:v>990</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -17894,13 +17888,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B74" s="1" t="s">
-        <x:v>1126</x:v>
+        <x:v>1124</x:v>
       </x:c>
       <x:c r="C74" s="1" t="s">
-        <x:v>1127</x:v>
+        <x:v>1125</x:v>
       </x:c>
       <x:c r="D74" s="1" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="3.9000000953674316" customHeight="1">
@@ -17908,10 +17902,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B75" s="1" t="s">
-        <x:v>1128</x:v>
+        <x:v>1126</x:v>
       </x:c>
       <x:c r="C75" s="1" t="s">
-        <x:v>1129</x:v>
+        <x:v>1127</x:v>
       </x:c>
       <x:c r="D75" s="1"/>
     </x:row>
@@ -17920,10 +17914,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B76" s="1" t="s">
-        <x:v>1130</x:v>
+        <x:v>1128</x:v>
       </x:c>
       <x:c r="C76" s="1" t="s">
-        <x:v>1131</x:v>
+        <x:v>1129</x:v>
       </x:c>
       <x:c r="D76" s="1"/>
     </x:row>
@@ -17932,10 +17926,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B77" s="1" t="s">
-        <x:v>1132</x:v>
+        <x:v>1130</x:v>
       </x:c>
       <x:c r="C77" s="1" t="s">
-        <x:v>1133</x:v>
+        <x:v>1131</x:v>
       </x:c>
       <x:c r="D77" s="1"/>
     </x:row>
@@ -17944,129 +17938,129 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B78" s="1" t="s">
-        <x:v>1134</x:v>
+        <x:v>1132</x:v>
       </x:c>
       <x:c r="C78" s="1" t="s">
-        <x:v>1135</x:v>
+        <x:v>1133</x:v>
       </x:c>
       <x:c r="D78" s="1"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="1" t="s">
+        <x:v>1134</x:v>
+      </x:c>
+      <x:c r="B79" s="1" t="s">
+        <x:v>1135</x:v>
+      </x:c>
+      <x:c r="C79" s="1" t="s">
         <x:v>1136</x:v>
-      </x:c>
-      <x:c r="B79" s="1" t="s">
-        <x:v>1137</x:v>
-      </x:c>
-      <x:c r="C79" s="1" t="s">
-        <x:v>1138</x:v>
       </x:c>
       <x:c r="D79" s="1"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="1" t="s">
-        <x:v>1136</x:v>
+        <x:v>1134</x:v>
       </x:c>
       <x:c r="B80" s="1" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="C80" s="1" t="s">
-        <x:v>1139</x:v>
+        <x:v>1137</x:v>
       </x:c>
       <x:c r="D80" s="1"/>
     </x:row>
     <x:row r="81" ht="3.9000000953674316" customHeight="1">
       <x:c r="A81" s="1" t="s">
+        <x:v>1138</x:v>
+      </x:c>
+      <x:c r="B81" s="1" t="s">
+        <x:v>1139</x:v>
+      </x:c>
+      <x:c r="C81" s="1" t="s">
         <x:v>1140</x:v>
-      </x:c>
-      <x:c r="B81" s="1" t="s">
-        <x:v>1141</x:v>
-      </x:c>
-      <x:c r="C81" s="1" t="s">
-        <x:v>1142</x:v>
       </x:c>
       <x:c r="D81" s="1"/>
     </x:row>
     <x:row r="82" ht="3.9000000953674316" customHeight="1">
       <x:c r="A82" s="1" t="s">
-        <x:v>1140</x:v>
+        <x:v>1138</x:v>
       </x:c>
       <x:c r="B82" s="1" t="s">
-        <x:v>1143</x:v>
+        <x:v>1141</x:v>
       </x:c>
       <x:c r="C82" s="1" t="s">
-        <x:v>1144</x:v>
+        <x:v>1142</x:v>
       </x:c>
       <x:c r="D82" s="1"/>
     </x:row>
     <x:row r="83" ht="3.9000000953674316" customHeight="1">
       <x:c r="A83" s="1" t="s">
-        <x:v>1140</x:v>
+        <x:v>1138</x:v>
       </x:c>
       <x:c r="B83" s="1" t="s">
-        <x:v>1145</x:v>
+        <x:v>1143</x:v>
       </x:c>
       <x:c r="C83" s="1" t="s">
-        <x:v>1146</x:v>
+        <x:v>1144</x:v>
       </x:c>
       <x:c r="D83" s="1"/>
     </x:row>
     <x:row r="84" ht="3.9000000953674316" customHeight="1">
       <x:c r="A84" s="1" t="s">
+        <x:v>1145</x:v>
+      </x:c>
+      <x:c r="B84" s="1" t="s">
+        <x:v>1146</x:v>
+      </x:c>
+      <x:c r="C84" s="1" t="s">
         <x:v>1147</x:v>
-      </x:c>
-      <x:c r="B84" s="1" t="s">
-        <x:v>1148</x:v>
-      </x:c>
-      <x:c r="C84" s="1" t="s">
-        <x:v>1149</x:v>
       </x:c>
       <x:c r="D84" s="1"/>
     </x:row>
     <x:row r="85" ht="3.9000000953674316" customHeight="1">
       <x:c r="A85" s="1" t="s">
-        <x:v>1147</x:v>
+        <x:v>1145</x:v>
       </x:c>
       <x:c r="B85" s="1" t="s">
-        <x:v>1150</x:v>
+        <x:v>1148</x:v>
       </x:c>
       <x:c r="C85" s="1" t="s">
-        <x:v>1151</x:v>
+        <x:v>1149</x:v>
       </x:c>
       <x:c r="D85" s="1"/>
     </x:row>
     <x:row r="86" ht="3.9000000953674316" customHeight="1">
       <x:c r="A86" s="1" t="s">
-        <x:v>1147</x:v>
+        <x:v>1145</x:v>
       </x:c>
       <x:c r="B86" s="1" t="s">
-        <x:v>1152</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="C86" s="1" t="s">
-        <x:v>1153</x:v>
+        <x:v>1151</x:v>
       </x:c>
       <x:c r="D86" s="1"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" t="s">
+        <x:v>1152</x:v>
+      </x:c>
+      <x:c r="B87" t="s">
+        <x:v>1153</x:v>
+      </x:c>
+      <x:c r="C87" t="s">
         <x:v>1154</x:v>
-      </x:c>
-      <x:c r="B87" t="s">
-        <x:v>1155</x:v>
-      </x:c>
-      <x:c r="C87" t="s">
-        <x:v>1156</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="s">
-        <x:v>1154</x:v>
+        <x:v>1152</x:v>
       </x:c>
       <x:c r="B88" t="s">
-        <x:v>1157</x:v>
+        <x:v>1155</x:v>
       </x:c>
       <x:c r="C88" t="s">
-        <x:v>1158</x:v>
+        <x:v>1156</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -18074,10 +18068,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B89" t="s">
-        <x:v>1159</x:v>
+        <x:v>1157</x:v>
       </x:c>
       <x:c r="C89" t="s">
-        <x:v>1160</x:v>
+        <x:v>1158</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -18085,10 +18079,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B90" t="s">
-        <x:v>1161</x:v>
+        <x:v>1159</x:v>
       </x:c>
       <x:c r="C90" t="s">
-        <x:v>1162</x:v>
+        <x:v>1160</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -18096,10 +18090,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B91" t="s">
-        <x:v>1163</x:v>
+        <x:v>1161</x:v>
       </x:c>
       <x:c r="C91" t="s">
-        <x:v>1164</x:v>
+        <x:v>1162</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -18107,10 +18101,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B92" t="s">
-        <x:v>1165</x:v>
+        <x:v>1163</x:v>
       </x:c>
       <x:c r="C92" t="s">
-        <x:v>1166</x:v>
+        <x:v>1164</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -18118,21 +18112,21 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B93" t="s">
-        <x:v>1167</x:v>
+        <x:v>1165</x:v>
       </x:c>
       <x:c r="C93" t="s">
-        <x:v>1168</x:v>
+        <x:v>1166</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" t="s">
+        <x:v>1167</x:v>
+      </x:c>
+      <x:c r="B94" t="s">
+        <x:v>1168</x:v>
+      </x:c>
+      <x:c r="C94" t="s">
         <x:v>1169</x:v>
-      </x:c>
-      <x:c r="B94" t="s">
-        <x:v>1170</x:v>
-      </x:c>
-      <x:c r="C94" t="s">
-        <x:v>1171</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18150,18 +18144,18 @@
   <x:sheetData>
     <x:row r="1" ht="3.9000000953674316" customHeight="1">
       <x:c r="A1" s="2" t="s">
-        <x:v>1172</x:v>
+        <x:v>1170</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>1173</x:v>
+        <x:v>1171</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="11.399999618530273" customHeight="1">
       <x:c r="A2" s="1" t="s">
-        <x:v>1174</x:v>
+        <x:v>1172</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>1175</x:v>
+        <x:v>1173</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18180,112 +18174,112 @@
   <x:sheetData>
     <x:row r="1" ht="3.9000000953674316" customHeight="1">
       <x:c r="A1" s="2" t="s">
+        <x:v>1174</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="s">
+        <x:v>1175</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="s">
         <x:v>1176</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="s">
-        <x:v>1177</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>1178</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="11.399999618530273" customHeight="1">
       <x:c r="A2" s="1" t="s">
+        <x:v>1177</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>1178</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
         <x:v>1179</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>1180</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>1181</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="7.650000095367432" customHeight="1">
       <x:c r="A3" s="1" t="s">
+        <x:v>1180</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="s">
+        <x:v>1181</x:v>
+      </x:c>
+      <x:c r="C3" s="1" t="s">
         <x:v>1182</x:v>
-      </x:c>
-      <x:c r="B3" s="1" t="s">
-        <x:v>1183</x:v>
-      </x:c>
-      <x:c r="C3" s="1" t="s">
-        <x:v>1184</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="7.650000095367432" customHeight="1">
       <x:c r="A4" s="1" t="s">
+        <x:v>1183</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="s">
+        <x:v>1184</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="s">
         <x:v>1185</x:v>
-      </x:c>
-      <x:c r="B4" s="1" t="s">
-        <x:v>1186</x:v>
-      </x:c>
-      <x:c r="C4" s="1" t="s">
-        <x:v>1187</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="13.399999618530273" customHeight="1">
       <x:c r="A5" s="1" t="s">
+        <x:v>1186</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="s">
+        <x:v>1187</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="s">
         <x:v>1188</x:v>
-      </x:c>
-      <x:c r="B5" s="1" t="s">
-        <x:v>1189</x:v>
-      </x:c>
-      <x:c r="C5" s="1" t="s">
-        <x:v>1190</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="9.649999618530273" customHeight="1">
       <x:c r="A6" s="1" t="s">
+        <x:v>1189</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="s">
+        <x:v>1190</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="s">
         <x:v>1191</x:v>
-      </x:c>
-      <x:c r="B6" s="1" t="s">
-        <x:v>1192</x:v>
-      </x:c>
-      <x:c r="C6" s="1" t="s">
-        <x:v>1193</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15.25" customHeight="1">
       <x:c r="A7" s="1" t="s">
+        <x:v>1192</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="s">
+        <x:v>1193</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="s">
         <x:v>1194</x:v>
-      </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>1195</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>1196</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15.25" customHeight="1">
       <x:c r="A8" s="1" t="s">
+        <x:v>1195</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="s">
+        <x:v>1196</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="s">
         <x:v>1197</x:v>
-      </x:c>
-      <x:c r="B8" s="1" t="s">
-        <x:v>1198</x:v>
-      </x:c>
-      <x:c r="C8" s="1" t="s">
-        <x:v>1199</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="19.149999618530273" customHeight="1">
       <x:c r="A9" s="1" t="s">
+        <x:v>1198</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="s">
+        <x:v>1199</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="s">
         <x:v>1200</x:v>
-      </x:c>
-      <x:c r="B9" s="1" t="s">
-        <x:v>1201</x:v>
-      </x:c>
-      <x:c r="C9" s="1" t="s">
-        <x:v>1202</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="17.149999618530273" customHeight="1">
       <x:c r="A10" s="1" t="s">
+        <x:v>1201</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="s">
+        <x:v>1202</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="s">
         <x:v>1203</x:v>
-      </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>1204</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="s">
-        <x:v>1205</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="11.399999618530273" customHeight="1">
@@ -18321,1107 +18315,1107 @@
   <x:sheetData>
     <x:row r="1" ht="3.9000000953674316" customHeight="1">
       <x:c r="A1" s="2" t="s">
+        <x:v>1204</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="s">
+        <x:v>1205</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="s">
         <x:v>1206</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="s">
+      <x:c r="D1" s="2" t="s">
         <x:v>1207</x:v>
       </x:c>
-      <x:c r="C1" s="2" t="s">
+      <x:c r="E1" s="2" t="s">
         <x:v>1208</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="s">
-        <x:v>1209</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="s">
-        <x:v>1210</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="47.75" customHeight="1">
       <x:c r="A2" s="1" t="s">
+        <x:v>1209</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>1210</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
         <x:v>1211</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
+      <x:c r="D2" s="1" t="s">
         <x:v>1212</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="E2" s="1" t="s">
         <x:v>1213</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>1214</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>1215</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="51.650001525878906" customHeight="1">
       <x:c r="A3" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B3" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
-        <x:v>1216</x:v>
+        <x:v>1214</x:v>
       </x:c>
       <x:c r="D3" s="1" t="s">
-        <x:v>1217</x:v>
+        <x:v>1215</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="53.400001525878906" customHeight="1">
       <x:c r="A4" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B4" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>1218</x:v>
+        <x:v>1216</x:v>
       </x:c>
       <x:c r="D4" s="1" t="s">
-        <x:v>1219</x:v>
+        <x:v>1217</x:v>
       </x:c>
       <x:c r="E4" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="53.900001525878906" customHeight="1">
       <x:c r="A5" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B5" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
-        <x:v>1220</x:v>
+        <x:v>1218</x:v>
       </x:c>
       <x:c r="D5" s="1" t="s">
-        <x:v>1221</x:v>
+        <x:v>1219</x:v>
       </x:c>
       <x:c r="E5" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="47.75" customHeight="1">
       <x:c r="A6" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B6" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>1222</x:v>
+        <x:v>1220</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>1223</x:v>
+        <x:v>1221</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="53.400001525878906" customHeight="1">
       <x:c r="A7" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>1224</x:v>
+        <x:v>1222</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>1225</x:v>
+        <x:v>1223</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="53.900001525878906" customHeight="1">
       <x:c r="A8" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>1226</x:v>
+        <x:v>1224</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>1227</x:v>
+        <x:v>1225</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="45.900001525878906" customHeight="1">
       <x:c r="A9" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>1228</x:v>
+        <x:v>1226</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>1229</x:v>
+        <x:v>1227</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="53.900001525878906" customHeight="1">
       <x:c r="A10" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>1230</x:v>
+        <x:v>1228</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>1231</x:v>
+        <x:v>1229</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="53.900001525878906" customHeight="1">
       <x:c r="A11" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>1232</x:v>
+        <x:v>1230</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>1233</x:v>
+        <x:v>1231</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="53.900001525878906" customHeight="1">
       <x:c r="A12" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B12" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>1234</x:v>
+        <x:v>1232</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
-        <x:v>1235</x:v>
+        <x:v>1233</x:v>
       </x:c>
       <x:c r="E12" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="53.900001525878906" customHeight="1">
       <x:c r="A13" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B13" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>1236</x:v>
+        <x:v>1234</x:v>
       </x:c>
       <x:c r="D13" s="1" t="s">
-        <x:v>1237</x:v>
+        <x:v>1235</x:v>
       </x:c>
       <x:c r="E13" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="53.900001525878906" customHeight="1">
       <x:c r="A14" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B14" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>1238</x:v>
+        <x:v>1236</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
-        <x:v>1239</x:v>
+        <x:v>1237</x:v>
       </x:c>
       <x:c r="E14" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="53.900001525878906" customHeight="1">
       <x:c r="A15" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B15" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>1240</x:v>
+        <x:v>1238</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
-        <x:v>1241</x:v>
+        <x:v>1239</x:v>
       </x:c>
       <x:c r="E15" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="53.900001525878906" customHeight="1">
       <x:c r="A16" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B16" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>1242</x:v>
+        <x:v>1240</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
-        <x:v>1243</x:v>
+        <x:v>1241</x:v>
       </x:c>
       <x:c r="E16" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28.649999618530273" customHeight="1">
       <x:c r="A17" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B17" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C17" s="1" t="s">
-        <x:v>1244</x:v>
+        <x:v>1242</x:v>
       </x:c>
       <x:c r="D17" s="1" t="s">
-        <x:v>1245</x:v>
+        <x:v>1243</x:v>
       </x:c>
       <x:c r="E17" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="28.649999618530273" customHeight="1">
       <x:c r="A18" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B18" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C18" s="1" t="s">
-        <x:v>1246</x:v>
+        <x:v>1244</x:v>
       </x:c>
       <x:c r="D18" s="1" t="s">
-        <x:v>1247</x:v>
+        <x:v>1245</x:v>
       </x:c>
       <x:c r="E18" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28.649999618530273" customHeight="1">
       <x:c r="A19" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B19" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C19" s="1" t="s">
-        <x:v>1248</x:v>
+        <x:v>1246</x:v>
       </x:c>
       <x:c r="D19" s="1" t="s">
-        <x:v>1249</x:v>
+        <x:v>1247</x:v>
       </x:c>
       <x:c r="E19" s="1" t="s">
-        <x:v>1215</x:v>
+        <x:v>1213</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28.649999618530273" customHeight="1">
       <x:c r="A20" s="1" t="s">
-        <x:v>1211</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
-        <x:v>1212</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
+        <x:v>1248</x:v>
+      </x:c>
+      <x:c r="D20" s="1" t="s">
+        <x:v>1249</x:v>
+      </x:c>
+      <x:c r="E20" s="1" t="s">
         <x:v>1250</x:v>
-      </x:c>
-      <x:c r="D20" s="1" t="s">
-        <x:v>1251</x:v>
-      </x:c>
-      <x:c r="E20" s="1" t="s">
-        <x:v>1252</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="28.649999618530273" customHeight="1">
       <x:c r="A21" s="1" t="s">
+        <x:v>1251</x:v>
+      </x:c>
+      <x:c r="B21" s="1" t="s">
+        <x:v>1252</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="s">
         <x:v>1253</x:v>
       </x:c>
-      <x:c r="B21" s="1" t="s">
+      <x:c r="D21" s="1" t="s">
         <x:v>1254</x:v>
       </x:c>
-      <x:c r="C21" s="1" t="s">
+      <x:c r="E21" s="1" t="s">
         <x:v>1255</x:v>
-      </x:c>
-      <x:c r="D21" s="1" t="s">
-        <x:v>1256</x:v>
-      </x:c>
-      <x:c r="E21" s="1" t="s">
-        <x:v>1257</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28.649999618530273" customHeight="1">
       <x:c r="A22" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>1258</x:v>
+        <x:v>1256</x:v>
       </x:c>
       <x:c r="D22" s="1" t="s">
-        <x:v>1259</x:v>
+        <x:v>1257</x:v>
       </x:c>
       <x:c r="E22" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="28.649999618530273" customHeight="1">
       <x:c r="A23" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C23" s="1" t="s">
-        <x:v>1260</x:v>
+        <x:v>1258</x:v>
       </x:c>
       <x:c r="D23" s="1" t="s">
-        <x:v>1261</x:v>
+        <x:v>1259</x:v>
       </x:c>
       <x:c r="E23" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="28.649999618530273" customHeight="1">
       <x:c r="A24" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C24" s="1" t="s">
-        <x:v>1262</x:v>
+        <x:v>1260</x:v>
       </x:c>
       <x:c r="D24" s="1" t="s">
-        <x:v>1263</x:v>
+        <x:v>1261</x:v>
       </x:c>
       <x:c r="E24" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28.649999618530273" customHeight="1">
       <x:c r="A25" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C25" s="1" t="s">
-        <x:v>1264</x:v>
+        <x:v>1262</x:v>
       </x:c>
       <x:c r="D25" s="1" t="s">
-        <x:v>1265</x:v>
+        <x:v>1263</x:v>
       </x:c>
       <x:c r="E25" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28.649999618530273" customHeight="1">
       <x:c r="A26" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C26" s="1" t="s">
-        <x:v>1266</x:v>
+        <x:v>1264</x:v>
       </x:c>
       <x:c r="D26" s="1" t="s">
-        <x:v>1267</x:v>
+        <x:v>1265</x:v>
       </x:c>
       <x:c r="E26" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="28.649999618530273" customHeight="1">
       <x:c r="A27" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
-        <x:v>1268</x:v>
+        <x:v>1266</x:v>
       </x:c>
       <x:c r="D27" s="1" t="s">
-        <x:v>1269</x:v>
+        <x:v>1267</x:v>
       </x:c>
       <x:c r="E27" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="28.649999618530273" customHeight="1">
       <x:c r="A28" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B28" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
-        <x:v>1270</x:v>
+        <x:v>1268</x:v>
       </x:c>
       <x:c r="D28" s="1" t="s">
-        <x:v>1271</x:v>
+        <x:v>1269</x:v>
       </x:c>
       <x:c r="E28" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="28.649999618530273" customHeight="1">
       <x:c r="A29" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
-        <x:v>1272</x:v>
+        <x:v>1270</x:v>
       </x:c>
       <x:c r="D29" s="1" t="s">
-        <x:v>1273</x:v>
+        <x:v>1271</x:v>
       </x:c>
       <x:c r="E29" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="28.649999618530273" customHeight="1">
       <x:c r="A30" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C30" s="1" t="s">
-        <x:v>1274</x:v>
+        <x:v>1272</x:v>
       </x:c>
       <x:c r="D30" s="1" t="s">
-        <x:v>1275</x:v>
+        <x:v>1273</x:v>
       </x:c>
       <x:c r="E30" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="28.649999618530273" customHeight="1">
       <x:c r="A31" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C31" s="1" t="s">
-        <x:v>1276</x:v>
+        <x:v>1274</x:v>
       </x:c>
       <x:c r="D31" s="1" t="s">
-        <x:v>1277</x:v>
+        <x:v>1275</x:v>
       </x:c>
       <x:c r="E31" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28.649999618530273" customHeight="1">
       <x:c r="A32" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B32" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C32" s="1" t="s">
-        <x:v>1278</x:v>
+        <x:v>1276</x:v>
       </x:c>
       <x:c r="D32" s="1" t="s">
-        <x:v>1279</x:v>
+        <x:v>1277</x:v>
       </x:c>
       <x:c r="E32" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28.649999618530273" customHeight="1">
       <x:c r="A33" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B33" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C33" s="1" t="s">
-        <x:v>1280</x:v>
+        <x:v>1278</x:v>
       </x:c>
       <x:c r="D33" s="1" t="s">
-        <x:v>1281</x:v>
+        <x:v>1279</x:v>
       </x:c>
       <x:c r="E33" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="28.649999618530273" customHeight="1">
       <x:c r="A34" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B34" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C34" s="1" t="s">
-        <x:v>1282</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="D34" s="1" t="s">
-        <x:v>1283</x:v>
+        <x:v>1281</x:v>
       </x:c>
       <x:c r="E34" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="28.649999618530273" customHeight="1">
       <x:c r="A35" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B35" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C35" s="1" t="s">
-        <x:v>1284</x:v>
+        <x:v>1282</x:v>
       </x:c>
       <x:c r="D35" s="1" t="s">
-        <x:v>1285</x:v>
+        <x:v>1283</x:v>
       </x:c>
       <x:c r="E35" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28.649999618530273" customHeight="1">
       <x:c r="A36" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B36" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C36" s="1" t="s">
-        <x:v>1286</x:v>
+        <x:v>1284</x:v>
       </x:c>
       <x:c r="D36" s="1" t="s">
-        <x:v>1287</x:v>
+        <x:v>1285</x:v>
       </x:c>
       <x:c r="E36" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28.649999618530273" customHeight="1">
       <x:c r="A37" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C37" s="1" t="s">
-        <x:v>1288</x:v>
+        <x:v>1286</x:v>
       </x:c>
       <x:c r="D37" s="1" t="s">
-        <x:v>1289</x:v>
+        <x:v>1287</x:v>
       </x:c>
       <x:c r="E37" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="28.649999618530273" customHeight="1">
       <x:c r="A38" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C38" s="1" t="s">
-        <x:v>1290</x:v>
+        <x:v>1288</x:v>
       </x:c>
       <x:c r="D38" s="1" t="s">
-        <x:v>1291</x:v>
+        <x:v>1289</x:v>
       </x:c>
       <x:c r="E38" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="28.649999618530273" customHeight="1">
       <x:c r="A39" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C39" s="1" t="s">
-        <x:v>1292</x:v>
+        <x:v>1290</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
-        <x:v>1293</x:v>
+        <x:v>1291</x:v>
       </x:c>
       <x:c r="E39" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="28.649999618530273" customHeight="1">
       <x:c r="A40" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C40" s="1" t="s">
-        <x:v>1294</x:v>
+        <x:v>1292</x:v>
       </x:c>
       <x:c r="D40" s="1" t="s">
-        <x:v>1295</x:v>
+        <x:v>1293</x:v>
       </x:c>
       <x:c r="E40" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28.649999618530273" customHeight="1">
       <x:c r="A41" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C41" s="1" t="s">
-        <x:v>1296</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="D41" s="1" t="s">
-        <x:v>1297</x:v>
+        <x:v>1295</x:v>
       </x:c>
       <x:c r="E41" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28.649999618530273" customHeight="1">
       <x:c r="A42" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B42" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C42" s="1" t="s">
-        <x:v>1298</x:v>
+        <x:v>1296</x:v>
       </x:c>
       <x:c r="D42" s="1" t="s">
-        <x:v>1299</x:v>
+        <x:v>1297</x:v>
       </x:c>
       <x:c r="E42" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="28.649999618530273" customHeight="1">
       <x:c r="A43" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B43" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C43" s="1" t="s">
-        <x:v>1300</x:v>
+        <x:v>1298</x:v>
       </x:c>
       <x:c r="D43" s="1" t="s">
-        <x:v>1301</x:v>
+        <x:v>1299</x:v>
       </x:c>
       <x:c r="E43" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="30.649999618530273" customHeight="1">
       <x:c r="A44" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B44" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C44" s="1" t="s">
-        <x:v>1302</x:v>
+        <x:v>1300</x:v>
       </x:c>
       <x:c r="D44" s="1" t="s">
-        <x:v>1303</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="E44" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28.649999618530273" customHeight="1">
       <x:c r="A45" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B45" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C45" s="1" t="s">
-        <x:v>1304</x:v>
+        <x:v>1302</x:v>
       </x:c>
       <x:c r="D45" s="1" t="s">
-        <x:v>1305</x:v>
+        <x:v>1303</x:v>
       </x:c>
       <x:c r="E45" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="28.649999618530273" customHeight="1">
       <x:c r="A46" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B46" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C46" s="1" t="s">
-        <x:v>1306</x:v>
+        <x:v>1304</x:v>
       </x:c>
       <x:c r="D46" s="1" t="s">
-        <x:v>1307</x:v>
+        <x:v>1305</x:v>
       </x:c>
       <x:c r="E46" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="28.649999618530273" customHeight="1">
       <x:c r="A47" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B47" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C47" s="1" t="s">
-        <x:v>1308</x:v>
+        <x:v>1306</x:v>
       </x:c>
       <x:c r="D47" s="1" t="s">
-        <x:v>1309</x:v>
+        <x:v>1307</x:v>
       </x:c>
       <x:c r="E47" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28.649999618530273" customHeight="1">
       <x:c r="A48" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B48" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C48" s="1" t="s">
-        <x:v>1310</x:v>
+        <x:v>1308</x:v>
       </x:c>
       <x:c r="D48" s="1" t="s">
-        <x:v>1311</x:v>
+        <x:v>1309</x:v>
       </x:c>
       <x:c r="E48" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28.649999618530273" customHeight="1">
       <x:c r="A49" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B49" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C49" s="1" t="s">
-        <x:v>1312</x:v>
+        <x:v>1310</x:v>
       </x:c>
       <x:c r="D49" s="1" t="s">
-        <x:v>1313</x:v>
+        <x:v>1311</x:v>
       </x:c>
       <x:c r="E49" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="28.649999618530273" customHeight="1">
       <x:c r="A50" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B50" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C50" s="1" t="s">
-        <x:v>1314</x:v>
+        <x:v>1312</x:v>
       </x:c>
       <x:c r="D50" s="1" t="s">
-        <x:v>1315</x:v>
+        <x:v>1313</x:v>
       </x:c>
       <x:c r="E50" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="28.649999618530273" customHeight="1">
       <x:c r="A51" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B51" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C51" s="1" t="s">
-        <x:v>1316</x:v>
+        <x:v>1314</x:v>
       </x:c>
       <x:c r="D51" s="1" t="s">
-        <x:v>1317</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="E51" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28.649999618530273" customHeight="1">
       <x:c r="A52" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B52" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C52" s="1" t="s">
-        <x:v>1318</x:v>
+        <x:v>1316</x:v>
       </x:c>
       <x:c r="D52" s="1" t="s">
-        <x:v>1319</x:v>
+        <x:v>1317</x:v>
       </x:c>
       <x:c r="E52" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28.649999618530273" customHeight="1">
       <x:c r="A53" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B53" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C53" s="1" t="s">
-        <x:v>1320</x:v>
+        <x:v>1318</x:v>
       </x:c>
       <x:c r="D53" s="1" t="s">
-        <x:v>1321</x:v>
+        <x:v>1319</x:v>
       </x:c>
       <x:c r="E53" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28.649999618530273" customHeight="1">
       <x:c r="A54" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B54" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C54" s="1" t="s">
-        <x:v>1322</x:v>
+        <x:v>1320</x:v>
       </x:c>
       <x:c r="D54" s="1" t="s">
-        <x:v>1323</x:v>
+        <x:v>1321</x:v>
       </x:c>
       <x:c r="E54" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B55" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C55" s="1" t="s">
-        <x:v>1324</x:v>
+        <x:v>1322</x:v>
       </x:c>
       <x:c r="D55" s="1" t="s">
-        <x:v>1325</x:v>
+        <x:v>1323</x:v>
       </x:c>
       <x:c r="E55" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="29">
       <x:c r="A56" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B56" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C56" s="1" t="s">
-        <x:v>1326</x:v>
+        <x:v>1324</x:v>
       </x:c>
       <x:c r="D56" s="1" t="s">
-        <x:v>1327</x:v>
+        <x:v>1325</x:v>
       </x:c>
       <x:c r="E56" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="29">
       <x:c r="A57" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B57" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C57" s="1" t="s">
-        <x:v>1328</x:v>
+        <x:v>1326</x:v>
       </x:c>
       <x:c r="D57" s="1" t="s">
-        <x:v>1329</x:v>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="E57" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="29">
       <x:c r="A58" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B58" s="1" t="s">
-        <x:v>1254</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C58" s="1" t="s">
-        <x:v>1330</x:v>
+        <x:v>1328</x:v>
       </x:c>
       <x:c r="D58" s="1" t="s">
-        <x:v>1331</x:v>
+        <x:v>1329</x:v>
       </x:c>
       <x:c r="E58" s="1" t="s">
-        <x:v>1257</x:v>
+        <x:v>1255</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B59" s="1" t="s">
+        <x:v>1330</x:v>
+      </x:c>
+      <x:c r="C59" s="1" t="s">
+        <x:v>1216</x:v>
+      </x:c>
+      <x:c r="D59" s="1" t="s">
+        <x:v>1331</x:v>
+      </x:c>
+      <x:c r="E59" s="1" t="s">
         <x:v>1332</x:v>
-      </x:c>
-      <x:c r="C59" s="1" t="s">
-        <x:v>1218</x:v>
-      </x:c>
-      <x:c r="D59" s="1" t="s">
-        <x:v>1333</x:v>
-      </x:c>
-      <x:c r="E59" s="1" t="s">
-        <x:v>1334</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1" t="s">
-        <x:v>1253</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="B60" s="1" t="s">
+        <x:v>1330</x:v>
+      </x:c>
+      <x:c r="C60" s="1" t="s">
+        <x:v>1333</x:v>
+      </x:c>
+      <x:c r="D60" s="1" t="s">
+        <x:v>1334</x:v>
+      </x:c>
+      <x:c r="E60" s="1" t="s">
         <x:v>1332</x:v>
-      </x:c>
-      <x:c r="C60" s="1" t="s">
-        <x:v>1335</x:v>
-      </x:c>
-      <x:c r="D60" s="1" t="s">
-        <x:v>1336</x:v>
-      </x:c>
-      <x:c r="E60" s="1" t="s">
-        <x:v>1334</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1" t="s">
-        <x:v>1337</x:v>
+        <x:v>1335</x:v>
       </x:c>
       <x:c r="B61" s="1" t="s">
-        <x:v>1338</x:v>
+        <x:v>1336</x:v>
       </x:c>
       <x:c r="C61" s="1" t="s">
-        <x:v>1156</x:v>
+        <x:v>1154</x:v>
       </x:c>
       <x:c r="D61" s="1" t="s">
         <x:v>959</x:v>
       </x:c>
       <x:c r="E61" s="1" t="s">
-        <x:v>1339</x:v>
+        <x:v>1337</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="1" t="s">
-        <x:v>1337</x:v>
+        <x:v>1335</x:v>
       </x:c>
       <x:c r="B62" s="1" t="s">
-        <x:v>1338</x:v>
+        <x:v>1336</x:v>
       </x:c>
       <x:c r="C62" s="1" t="s">
-        <x:v>1158</x:v>
+        <x:v>1156</x:v>
       </x:c>
       <x:c r="D62" s="1" t="s">
         <x:v>963</x:v>
       </x:c>
       <x:c r="E62" s="1" t="s">
-        <x:v>1339</x:v>
+        <x:v>1337</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1" t="s">
+        <x:v>1338</x:v>
+      </x:c>
+      <x:c r="B63" s="1" t="s">
+        <x:v>1339</x:v>
+      </x:c>
+      <x:c r="C63" s="1" t="s">
         <x:v>1340</x:v>
       </x:c>
-      <x:c r="B63" s="1" t="s">
+      <x:c r="D63" s="1" t="s">
+        <x:v>970</x:v>
+      </x:c>
+      <x:c r="E63" s="1" t="s">
         <x:v>1341</x:v>
-      </x:c>
-      <x:c r="C63" s="1" t="s">
-        <x:v>1342</x:v>
-      </x:c>
-      <x:c r="D63" s="1" t="s">
-        <x:v>972</x:v>
-      </x:c>
-      <x:c r="E63" s="1" t="s">
-        <x:v>1343</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1" t="s">
-        <x:v>1340</x:v>
+        <x:v>1338</x:v>
       </x:c>
       <x:c r="B64" s="1" t="s">
-        <x:v>1341</x:v>
+        <x:v>1339</x:v>
       </x:c>
       <x:c r="C64" s="1" t="s">
-        <x:v>1344</x:v>
+        <x:v>1342</x:v>
       </x:c>
       <x:c r="D64" s="1" t="s">
-        <x:v>974</x:v>
+        <x:v>972</x:v>
       </x:c>
       <x:c r="E64" s="1" t="s">
-        <x:v>1345</x:v>
+        <x:v>1343</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" t="s">
-        <x:v>1340</x:v>
+        <x:v>1338</x:v>
       </x:c>
       <x:c r="B65" t="s">
-        <x:v>1341</x:v>
+        <x:v>1339</x:v>
       </x:c>
       <x:c r="C65" t="s">
-        <x:v>979</x:v>
+        <x:v>977</x:v>
       </x:c>
       <x:c r="D65" t="s">
-        <x:v>978</x:v>
+        <x:v>976</x:v>
       </x:c>
       <x:c r="E65" t="s">
-        <x:v>1345</x:v>
+        <x:v>1343</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Force active GT HORECA templates and Kobo form
</commit_message>
<xml_diff>
--- a/templates/KB_Market_Improvement_XLSForm.xlsx
+++ b/templates/KB_Market_Improvement_XLSForm.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R656fd06bac004168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Re1688679d57a425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rd6e944611b654d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="R9595ba678a004b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="R99663956829847bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R044aa7db4e3046bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Ra4c39ed1d35e4b36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R464e73a2e02a4d0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="Rfb1a8fa6ff374df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="R2ac020d450774bb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -754,9 +754,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Calibri Light"/>
-        <a:cs typeface="Calibri Light"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -942,7 +942,7 @@
         <x:v>Region</x:v>
       </x:c>
       <x:c r="D3" s="11" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="E3" s="11" t="str">
         <x:v>ជ្រើសរើស Region</x:v>
@@ -967,7 +967,7 @@
         <x:v>Dealer</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
         <x:v>Dealer list filters by Region</x:v>
@@ -1019,14 +1019,12 @@
         <x:v>Report Date</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="E6" s="11"/>
       <x:c r="F6" s="11"/>
       <x:c r="G6" s="11"/>
-      <x:c r="H6" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H6" s="11"/>
       <x:c r="I6" s="11"/>
       <x:c r="J6" s="11"/>
       <x:c r="K6" s="11"/>
@@ -1047,9 +1045,7 @@
       <x:c r="E7" s="11"/>
       <x:c r="F7" s="11"/>
       <x:c r="G7" s="11"/>
-      <x:c r="H7" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H7" s="11"/>
       <x:c r="I7" s="11" t="str">
         <x:v>. &gt;= 0</x:v>
       </x:c>
@@ -1074,9 +1070,7 @@
       <x:c r="E8" s="11"/>
       <x:c r="F8" s="11"/>
       <x:c r="G8" s="11"/>
-      <x:c r="H8" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H8" s="11"/>
       <x:c r="I8" s="11" t="str">
         <x:v>. &gt;= 0</x:v>
       </x:c>
@@ -1103,9 +1097,7 @@
       </x:c>
       <x:c r="F9" s="11"/>
       <x:c r="G9" s="11"/>
-      <x:c r="H9" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H9" s="11"/>
       <x:c r="I9" s="11"/>
       <x:c r="J9" s="11"/>
       <x:c r="K9" s="11"/>
@@ -1129,7 +1121,7 @@
       <x:c r="F10" s="11"/>
       <x:c r="G10" s="11"/>
       <x:c r="H10" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I10" s="11"/>
       <x:c r="J10" s="11"/>
@@ -1152,7 +1144,7 @@
       <x:c r="F11" s="11"/>
       <x:c r="G11" s="11"/>
       <x:c r="H11" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I11" s="11"/>
       <x:c r="J11" s="11"/>
@@ -1177,7 +1169,7 @@
       <x:c r="F12" s="11"/>
       <x:c r="G12" s="11"/>
       <x:c r="H12" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I12" s="11"/>
       <x:c r="J12" s="11"/>
@@ -1204,7 +1196,7 @@
       <x:c r="F13" s="11"/>
       <x:c r="G13" s="11"/>
       <x:c r="H13" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I13" s="11"/>
       <x:c r="J13" s="11"/>
@@ -1229,7 +1221,7 @@
       <x:c r="F14" s="11"/>
       <x:c r="G14" s="11"/>
       <x:c r="H14" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I14" s="11"/>
       <x:c r="J14" s="11"/>
@@ -1258,7 +1250,7 @@
         <x:v>contains(report_scope, ${final_summary_report_type})</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I15" s="11"/>
       <x:c r="J15" s="11"/>
@@ -1285,7 +1277,7 @@
       </x:c>
       <x:c r="G16" s="11"/>
       <x:c r="H16" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I16" s="11"/>
       <x:c r="J16" s="11"/>
@@ -1309,9 +1301,7 @@
       </x:c>
       <x:c r="F17" s="11"/>
       <x:c r="G17" s="11"/>
-      <x:c r="H17" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H17" s="11"/>
       <x:c r="I17" s="11"/>
       <x:c r="J17" s="11"/>
       <x:c r="K17" s="11"/>
@@ -1350,7 +1340,7 @@
       <x:c r="F19" s="11"/>
       <x:c r="G19" s="11"/>
       <x:c r="H19" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I19" s="11"/>
       <x:c r="J19" s="11"/>
@@ -2803,9 +2793,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G79" s="11"/>
-      <x:c r="H79" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H79" s="11"/>
       <x:c r="I79" s="11"/>
       <x:c r="J79" s="11"/>
       <x:c r="K79" s="11"/>
@@ -3094,9 +3082,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G90" s="11"/>
-      <x:c r="H90" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H90" s="11"/>
       <x:c r="I90" s="11"/>
       <x:c r="J90" s="11"/>
       <x:c r="K90" s="11"/>
@@ -3275,9 +3261,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G97" s="11"/>
-      <x:c r="H97" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H97" s="11"/>
       <x:c r="I97" s="11"/>
       <x:c r="J97" s="11"/>
       <x:c r="K97" s="11"/>
@@ -3456,9 +3440,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G104" s="11"/>
-      <x:c r="H104" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H104" s="11"/>
       <x:c r="I104" s="11"/>
       <x:c r="J104" s="11"/>
       <x:c r="K104" s="11"/>
@@ -3637,9 +3619,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G111" s="11"/>
-      <x:c r="H111" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H111" s="11"/>
       <x:c r="I111" s="11"/>
       <x:c r="J111" s="11"/>
       <x:c r="K111" s="11"/>
@@ -3928,9 +3908,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G122" s="11"/>
-      <x:c r="H122" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H122" s="11"/>
       <x:c r="I122" s="11"/>
       <x:c r="J122" s="11"/>
       <x:c r="K122" s="11"/>
@@ -4220,7 +4198,7 @@
       </x:c>
       <x:c r="G133" s="11"/>
       <x:c r="H133" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I133" s="11"/>
       <x:c r="J133" s="11"/>
@@ -4510,9 +4488,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G144" s="11"/>
-      <x:c r="H144" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H144" s="11"/>
       <x:c r="I144" s="11"/>
       <x:c r="J144" s="11"/>
       <x:c r="K144" s="11"/>
@@ -4691,9 +4667,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G151" s="11"/>
-      <x:c r="H151" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H151" s="11"/>
       <x:c r="I151" s="11"/>
       <x:c r="J151" s="11"/>
       <x:c r="K151" s="11"/>
@@ -4872,9 +4846,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G158" s="11"/>
-      <x:c r="H158" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H158" s="11"/>
       <x:c r="I158" s="11"/>
       <x:c r="J158" s="11"/>
       <x:c r="K158" s="11"/>
@@ -5053,9 +5025,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G165" s="11"/>
-      <x:c r="H165" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H165" s="11"/>
       <x:c r="I165" s="11"/>
       <x:c r="J165" s="11"/>
       <x:c r="K165" s="11"/>
@@ -5234,9 +5204,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G172" s="11"/>
-      <x:c r="H172" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H172" s="11"/>
       <x:c r="I172" s="11"/>
       <x:c r="J172" s="11"/>
       <x:c r="K172" s="11"/>
@@ -5415,9 +5383,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G179" s="11"/>
-      <x:c r="H179" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H179" s="11"/>
       <x:c r="I179" s="11"/>
       <x:c r="J179" s="11"/>
       <x:c r="K179" s="11"/>
@@ -5596,9 +5562,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G186" s="11"/>
-      <x:c r="H186" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H186" s="11"/>
       <x:c r="I186" s="11"/>
       <x:c r="J186" s="11"/>
       <x:c r="K186" s="11"/>
@@ -5887,9 +5851,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G197" s="11"/>
-      <x:c r="H197" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H197" s="11"/>
       <x:c r="I197" s="11"/>
       <x:c r="J197" s="11"/>
       <x:c r="K197" s="11"/>
@@ -6089,9 +6051,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G205" s="11"/>
-      <x:c r="H205" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H205" s="11"/>
       <x:c r="I205" s="11"/>
       <x:c r="J205" s="11"/>
       <x:c r="K205" s="11"/>
@@ -6351,9 +6311,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G215" s="11"/>
-      <x:c r="H215" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H215" s="11"/>
       <x:c r="I215" s="11"/>
       <x:c r="J215" s="11"/>
       <x:c r="K215" s="11"/>
@@ -6628,9 +6586,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G226" s="11"/>
-      <x:c r="H226" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H226" s="11"/>
       <x:c r="I226" s="11"/>
       <x:c r="J226" s="11"/>
       <x:c r="K226" s="11"/>
@@ -6890,9 +6846,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G236" s="11"/>
-      <x:c r="H236" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H236" s="11"/>
       <x:c r="I236" s="11"/>
       <x:c r="J236" s="11"/>
       <x:c r="K236" s="11"/>
@@ -7071,9 +7025,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G243" s="11"/>
-      <x:c r="H243" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H243" s="11"/>
       <x:c r="I243" s="11"/>
       <x:c r="J243" s="11"/>
       <x:c r="K243" s="11"/>
@@ -7252,9 +7204,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G250" s="11"/>
-      <x:c r="H250" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H250" s="11"/>
       <x:c r="I250" s="11"/>
       <x:c r="J250" s="11"/>
       <x:c r="K250" s="11"/>
@@ -7515,7 +7465,7 @@
       </x:c>
       <x:c r="G260" s="11"/>
       <x:c r="H260" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I260" s="11"/>
       <x:c r="J260" s="11"/>
@@ -7696,7 +7646,7 @@
       </x:c>
       <x:c r="G267" s="11"/>
       <x:c r="H267" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I267" s="11"/>
       <x:c r="J267" s="11"/>
@@ -7877,7 +7827,7 @@
       </x:c>
       <x:c r="G274" s="11"/>
       <x:c r="H274" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I274" s="11"/>
       <x:c r="J274" s="11"/>
@@ -8057,9 +8007,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G281" s="11"/>
-      <x:c r="H281" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H281" s="11"/>
       <x:c r="I281" s="11"/>
       <x:c r="J281" s="11"/>
       <x:c r="K281" s="11"/>
@@ -8319,9 +8267,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G291" s="11"/>
-      <x:c r="H291" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H291" s="11"/>
       <x:c r="I291" s="11"/>
       <x:c r="J291" s="11"/>
       <x:c r="K291" s="11"/>
@@ -8500,9 +8446,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G298" s="11"/>
-      <x:c r="H298" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H298" s="11"/>
       <x:c r="I298" s="11"/>
       <x:c r="J298" s="11"/>
       <x:c r="K298" s="11"/>
@@ -8681,9 +8625,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G305" s="11"/>
-      <x:c r="H305" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H305" s="11"/>
       <x:c r="I305" s="11"/>
       <x:c r="J305" s="11"/>
       <x:c r="K305" s="11"/>
@@ -8943,9 +8885,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G315" s="11"/>
-      <x:c r="H315" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H315" s="11"/>
       <x:c r="I315" s="11"/>
       <x:c r="J315" s="11"/>
       <x:c r="K315" s="11"/>
@@ -11177,9 +11117,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G401" s="11"/>
-      <x:c r="H401" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H401" s="11"/>
       <x:c r="I401" s="11"/>
       <x:c r="J401" s="11"/>
       <x:c r="K401" s="11"/>
@@ -11439,9 +11377,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G411" s="11"/>
-      <x:c r="H411" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H411" s="11"/>
       <x:c r="I411" s="11"/>
       <x:c r="J411" s="11"/>
       <x:c r="K411" s="11"/>
@@ -11620,9 +11556,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G418" s="11"/>
-      <x:c r="H418" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H418" s="11"/>
       <x:c r="I418" s="11"/>
       <x:c r="J418" s="11"/>
       <x:c r="K418" s="11"/>
@@ -11801,9 +11735,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G425" s="11"/>
-      <x:c r="H425" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H425" s="11"/>
       <x:c r="I425" s="11"/>
       <x:c r="J425" s="11"/>
       <x:c r="K425" s="11"/>
@@ -11982,9 +11914,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G432" s="11"/>
-      <x:c r="H432" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H432" s="11"/>
       <x:c r="I432" s="11"/>
       <x:c r="J432" s="11"/>
       <x:c r="K432" s="11"/>
@@ -12244,9 +12174,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G442" s="11"/>
-      <x:c r="H442" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H442" s="11"/>
       <x:c r="I442" s="11"/>
       <x:c r="J442" s="11"/>
       <x:c r="K442" s="11"/>
@@ -12506,9 +12434,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G452" s="11"/>
-      <x:c r="H452" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H452" s="11"/>
       <x:c r="I452" s="11"/>
       <x:c r="J452" s="11"/>
       <x:c r="K452" s="11"/>
@@ -12687,9 +12613,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G459" s="11"/>
-      <x:c r="H459" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H459" s="11"/>
       <x:c r="I459" s="11"/>
       <x:c r="J459" s="11"/>
       <x:c r="K459" s="11"/>
@@ -12889,9 +12813,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G467" s="11"/>
-      <x:c r="H467" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H467" s="11"/>
       <x:c r="I467" s="11"/>
       <x:c r="J467" s="11"/>
       <x:c r="K467" s="11"/>
@@ -13151,9 +13073,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G477" s="11"/>
-      <x:c r="H477" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H477" s="11"/>
       <x:c r="I477" s="11"/>
       <x:c r="J477" s="11"/>
       <x:c r="K477" s="11"/>
@@ -13332,9 +13252,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G484" s="11"/>
-      <x:c r="H484" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H484" s="11"/>
       <x:c r="I484" s="11"/>
       <x:c r="J484" s="11"/>
       <x:c r="K484" s="11"/>
@@ -13513,9 +13431,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G491" s="11"/>
-      <x:c r="H491" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H491" s="11"/>
       <x:c r="I491" s="11"/>
       <x:c r="J491" s="11"/>
       <x:c r="K491" s="11"/>
@@ -13694,9 +13610,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G498" s="11"/>
-      <x:c r="H498" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H498" s="11"/>
       <x:c r="I498" s="11"/>
       <x:c r="J498" s="11"/>
       <x:c r="K498" s="11"/>
@@ -14879,7 +14793,7 @@
       </x:c>
       <x:c r="G544" s="11"/>
       <x:c r="H544" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
+        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
       </x:c>
       <x:c r="I544" s="11"/>
       <x:c r="J544" s="11"/>
@@ -14999,9 +14913,7 @@
       <x:c r="E549" s="11"/>
       <x:c r="F549" s="11"/>
       <x:c r="G549" s="11"/>
-      <x:c r="H549" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
-      </x:c>
+      <x:c r="H549" s="11"/>
       <x:c r="I549" s="11"/>
       <x:c r="J549" s="11"/>
       <x:c r="K549" s="11"/>

</xml_diff>